<commit_message>
EX1- fault analysis table update
</commit_message>
<xml_diff>
--- a/EX1/CPa_Fault_identification-analysis/EX1_CPa_All_models_confusion_matrix.xlsx
+++ b/EX1/CPa_Fault_identification-analysis/EX1_CPa_All_models_confusion_matrix.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xhulj\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xhulj\Desktop\CPa\EX1\CPa_Fault_identification-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC1AD86-7BB6-4DA4-B49E-3AE9CE8F2FF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F111D924-B8EE-4AF3-970C-B66F9CA399D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CodeBERT" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="48">
   <si>
     <t>QT</t>
   </si>
@@ -170,10 +170,67 @@
     <t>Cpa (alpha 0.15)</t>
   </si>
   <si>
-    <t>OS</t>
+    <t># faults identified</t>
   </si>
   <si>
-    <t># faults identified</t>
+    <r>
+      <t xml:space="preserve">QT </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(181 faulty code changes)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">OS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(163 faulty code changes)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">QT </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(695 faulty code changes)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">OS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(875 faulty code changes)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -357,7 +414,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -412,54 +469,26 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -480,11 +509,21 @@
     <xf numFmtId="1" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -775,53 +814,52 @@
     <col min="4" max="4" width="18.44140625" customWidth="1"/>
     <col min="5" max="5" width="8.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="7.88671875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="7.88671875" style="35" customWidth="1"/>
+    <col min="7" max="8" width="7.88671875" style="1" customWidth="1"/>
     <col min="9" max="9" width="7.21875" style="1" customWidth="1"/>
     <col min="10" max="10" width="8.33203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="33.21875" style="61" customWidth="1"/>
-    <col min="12" max="12" width="17" style="61" customWidth="1"/>
+    <col min="11" max="11" width="33.21875" style="47" customWidth="1"/>
+    <col min="12" max="12" width="17" style="47" customWidth="1"/>
     <col min="13" max="13" width="8.33203125" style="1" customWidth="1"/>
     <col min="14" max="14" width="16.6640625" style="1" customWidth="1"/>
     <col min="15" max="15" width="20.33203125" customWidth="1"/>
-    <col min="16" max="16" width="3.6640625" style="52" customWidth="1"/>
+    <col min="16" max="16" width="3.6640625" style="40" customWidth="1"/>
     <col min="17" max="17" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="8.6640625" customWidth="1"/>
-    <col min="23" max="23" width="8.77734375" style="37"/>
-    <col min="26" max="26" width="17.88671875" style="61" customWidth="1"/>
-    <col min="27" max="27" width="15.109375" style="61" customWidth="1"/>
+    <col min="23" max="23" width="8.77734375"/>
+    <col min="26" max="26" width="17.88671875" style="47" customWidth="1"/>
+    <col min="27" max="27" width="15.109375" style="47" customWidth="1"/>
     <col min="28" max="28" width="8.33203125" style="1" customWidth="1"/>
     <col min="29" max="29" width="16.6640625" style="1" customWidth="1"/>
     <col min="30" max="30" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="52" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="53" t="s">
+    <row r="1" spans="1:30" s="40" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="Q1" s="53" t="s">
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="Q1" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="53"/>
-      <c r="S1" s="53"/>
-      <c r="T1" s="53"/>
-      <c r="Z1" s="54"/>
-      <c r="AA1" s="54"/>
-      <c r="AB1" s="56"/>
-      <c r="AC1" s="56"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="59"/>
+      <c r="Z1" s="41"/>
+      <c r="AA1" s="41"/>
+      <c r="AB1" s="43"/>
+      <c r="AC1" s="43"/>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
@@ -840,21 +878,21 @@
         <v>6</v>
       </c>
       <c r="G2" s="3"/>
-      <c r="H2" s="42"/>
+      <c r="H2" s="35"/>
       <c r="I2" s="23" t="s">
         <v>17</v>
       </c>
       <c r="J2" s="20"/>
-      <c r="K2" s="60" t="s">
+      <c r="K2" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="67" t="s">
+      <c r="L2" s="53" t="s">
         <v>28</v>
       </c>
       <c r="M2" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="N2" s="57"/>
+      <c r="N2" s="20"/>
       <c r="Q2" s="2" t="s">
         <v>2</v>
       </c>
@@ -871,21 +909,21 @@
         <v>6</v>
       </c>
       <c r="V2" s="3"/>
-      <c r="W2" s="42"/>
+      <c r="W2" s="35"/>
       <c r="X2" s="23" t="s">
         <v>17</v>
       </c>
       <c r="Y2" s="20"/>
-      <c r="Z2" s="60" t="s">
+      <c r="Z2" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="AA2" s="67" t="s">
+      <c r="AA2" s="53" t="s">
         <v>28</v>
       </c>
       <c r="AB2" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="AC2" s="57"/>
+      <c r="AC2" s="20"/>
     </row>
     <row r="3" spans="1:30" ht="21.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
@@ -912,15 +950,15 @@
         <v>2354.96</v>
       </c>
       <c r="J3" s="24"/>
-      <c r="K3" s="60">
+      <c r="K3" s="46">
         <f>B3+D3</f>
         <v>92.41</v>
       </c>
-      <c r="L3" s="60">
+      <c r="L3" s="46">
         <f>B3</f>
         <v>28.67</v>
       </c>
-      <c r="M3" s="65">
+      <c r="M3" s="51">
         <f>L3/K3</f>
         <v>0.31024780867871443</v>
       </c>
@@ -946,15 +984,15 @@
         <f>SUM(Q3:R3)</f>
         <v>1143.68</v>
       </c>
-      <c r="Z3" s="60">
+      <c r="Z3" s="46">
         <f>Q3+S3</f>
         <v>90.11</v>
       </c>
-      <c r="AA3" s="60">
+      <c r="AA3" s="46">
         <f>Q3</f>
         <v>32.74</v>
       </c>
-      <c r="AB3" s="65">
+      <c r="AB3" s="51">
         <f>AA3/Z3</f>
         <v>0.36333370325158143</v>
       </c>
@@ -969,11 +1007,11 @@
       <c r="E4" s="5"/>
       <c r="I4" s="24"/>
       <c r="J4" s="24"/>
-      <c r="K4" s="60">
+      <c r="K4" s="46">
         <f>C3+E3</f>
         <v>2478.59</v>
       </c>
-      <c r="L4" s="60">
+      <c r="L4" s="46">
         <f>E3</f>
         <v>152.30000000000001</v>
       </c>
@@ -981,7 +1019,7 @@
         <f>L4/K4</f>
         <v>6.1446225474967621E-2</v>
       </c>
-      <c r="N4" s="65"/>
+      <c r="N4" s="51"/>
       <c r="O4" s="11"/>
       <c r="Q4" s="5"/>
       <c r="R4" s="5"/>
@@ -989,11 +1027,11 @@
       <c r="T4" s="5"/>
       <c r="U4" s="1"/>
       <c r="X4" s="9"/>
-      <c r="Z4" s="60">
+      <c r="Z4" s="46">
         <f>R3+T3</f>
         <v>1240.8900000000001</v>
       </c>
-      <c r="AA4" s="60">
+      <c r="AA4" s="46">
         <f>T3</f>
         <v>129.94999999999999</v>
       </c>
@@ -1001,7 +1039,7 @@
         <f>AA4/Z4</f>
         <v>0.10472322284811705</v>
       </c>
-      <c r="AC4" s="65"/>
+      <c r="AC4" s="51"/>
       <c r="AD4" s="11"/>
     </row>
     <row r="5" spans="1:30" ht="12.6" customHeight="1" x14ac:dyDescent="0.35">
@@ -1012,8 +1050,8 @@
       <c r="E5" s="5"/>
       <c r="I5" s="24"/>
       <c r="J5" s="24"/>
-      <c r="K5" s="60"/>
-      <c r="L5" s="60"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="46"/>
       <c r="M5" s="24"/>
       <c r="N5" s="24"/>
       <c r="O5" s="11"/>
@@ -1023,27 +1061,27 @@
       <c r="T5" s="5"/>
       <c r="U5" s="1"/>
       <c r="X5" s="9"/>
-      <c r="Z5" s="60"/>
-      <c r="AA5" s="60"/>
+      <c r="Z5" s="46"/>
+      <c r="AA5" s="46"/>
       <c r="AB5" s="24"/>
       <c r="AC5" s="24"/>
       <c r="AD5" s="11"/>
     </row>
     <row r="6" spans="1:30" ht="16.8" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4"/>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
       <c r="F6" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="36" t="s">
+      <c r="H6" s="13" t="s">
         <v>18</v>
       </c>
       <c r="I6" s="3" t="s">
@@ -1052,28 +1090,28 @@
       <c r="J6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K6" s="67" t="s">
+      <c r="K6" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="L6" s="67" t="s">
+      <c r="L6" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="M6" s="58"/>
-      <c r="N6" s="58"/>
+      <c r="M6" s="44"/>
+      <c r="N6" s="44"/>
       <c r="O6" s="11"/>
-      <c r="Q6" s="33" t="s">
+      <c r="Q6" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="R6" s="33"/>
-      <c r="S6" s="33"/>
-      <c r="T6" s="33"/>
+      <c r="R6" s="60"/>
+      <c r="S6" s="60"/>
+      <c r="T6" s="60"/>
       <c r="U6" s="3" t="s">
         <v>24</v>
       </c>
       <c r="V6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="W6" s="36" t="s">
+      <c r="W6" s="13" t="s">
         <v>18</v>
       </c>
       <c r="X6" s="3" t="s">
@@ -1082,38 +1120,38 @@
       <c r="Y6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="Z6" s="67" t="s">
+      <c r="Z6" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="AA6" s="67"/>
-      <c r="AB6" s="58"/>
-      <c r="AC6" s="58"/>
+      <c r="AA6" s="53"/>
+      <c r="AB6" s="44"/>
+      <c r="AC6" s="44"/>
       <c r="AD6" s="11"/>
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="K7" s="61" t="s">
+      <c r="K7" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="L7" s="67" t="s">
+      <c r="L7" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="M7" s="55" t="s">
+      <c r="M7" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="N7" s="55"/>
-      <c r="Z7" s="61" t="s">
+      <c r="N7" s="42"/>
+      <c r="Z7" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="AA7" s="67" t="s">
+      <c r="AA7" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="AB7" s="55" t="s">
+      <c r="AB7" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="AC7" s="55"/>
+      <c r="AC7" s="42"/>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -1139,7 +1177,7 @@
         <f>F8/F3</f>
         <v>0.88259043173862306</v>
       </c>
-      <c r="H8" s="43">
+      <c r="H8" s="36">
         <f>I8/F8</f>
         <v>0.94755722432287126</v>
       </c>
@@ -1147,23 +1185,23 @@
         <f>SUM(B8:C8)</f>
         <v>2150.14</v>
       </c>
-      <c r="J8" s="55">
+      <c r="J8" s="42">
         <f>I8/I3</f>
         <v>0.91302612358596313</v>
       </c>
-      <c r="K8" s="63">
+      <c r="K8" s="49">
         <f>B8+D8</f>
         <v>23.14</v>
       </c>
-      <c r="L8" s="63">
+      <c r="L8" s="49">
         <f>B8</f>
         <v>10.14</v>
       </c>
-      <c r="M8" s="65">
+      <c r="M8" s="51">
         <f>L8/K8</f>
         <v>0.43820224719101125</v>
       </c>
-      <c r="N8" s="65"/>
+      <c r="N8" s="51"/>
       <c r="Q8" s="12">
         <v>6</v>
       </c>
@@ -1184,7 +1222,7 @@
         <f>U8/U3</f>
         <v>0.72652141247182567</v>
       </c>
-      <c r="W8" s="41">
+      <c r="W8" s="34">
         <f>X8/U8</f>
         <v>0.92967942088934852</v>
       </c>
@@ -1196,19 +1234,19 @@
         <f>X8/X3</f>
         <v>0.78605903749300499</v>
       </c>
-      <c r="Z8" s="63">
+      <c r="Z8" s="49">
         <f>Q8+S8</f>
         <v>12</v>
       </c>
-      <c r="AA8" s="63">
+      <c r="AA8" s="49">
         <f>Q8</f>
         <v>6</v>
       </c>
-      <c r="AB8" s="65">
+      <c r="AB8" s="51">
         <f>AA8/Z8</f>
         <v>0.5</v>
       </c>
-      <c r="AC8" s="65"/>
+      <c r="AC8" s="51"/>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -1234,7 +1272,7 @@
         <f>F9/F3</f>
         <v>0.9743990665110851</v>
       </c>
-      <c r="H9" s="43">
+      <c r="H9" s="36">
         <f>I9/F9</f>
         <v>0.92615301096128821</v>
       </c>
@@ -1246,19 +1284,19 @@
         <f>I9/I3</f>
         <v>0.98523117165472018</v>
       </c>
-      <c r="K9" s="63">
+      <c r="K9" s="49">
         <f>B9+D9</f>
         <v>66.180000000000007</v>
       </c>
-      <c r="L9" s="63">
+      <c r="L9" s="49">
         <f>B9</f>
         <v>21.18</v>
       </c>
-      <c r="M9" s="65">
+      <c r="M9" s="51">
         <f>L9/K9</f>
         <v>0.32003626473254754</v>
       </c>
-      <c r="N9" s="65"/>
+      <c r="N9" s="51"/>
       <c r="Q9" s="12">
         <v>15</v>
       </c>
@@ -1279,7 +1317,7 @@
         <f>U9/U3</f>
         <v>0.92186326070623592</v>
       </c>
-      <c r="W9" s="41">
+      <c r="W9" s="34">
         <f>X9/U9</f>
         <v>0.88916055419722906</v>
       </c>
@@ -1291,19 +1329,19 @@
         <f>X9/X3</f>
         <v>0.95393816452154445</v>
       </c>
-      <c r="Z9" s="63">
+      <c r="Z9" s="49">
         <f>Q9+S9</f>
         <v>36</v>
       </c>
-      <c r="AA9" s="63">
+      <c r="AA9" s="49">
         <f>Q9</f>
         <v>15</v>
       </c>
-      <c r="AB9" s="65">
+      <c r="AB9" s="51">
         <f>AA9/Z9</f>
         <v>0.41666666666666669</v>
       </c>
-      <c r="AC9" s="65"/>
+      <c r="AC9" s="51"/>
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -1329,7 +1367,7 @@
         <f>F10/F3</f>
         <v>0.89977829638273044</v>
       </c>
-      <c r="H10" s="43">
+      <c r="H10" s="36">
         <f>I10/F10</f>
         <v>0.94423623088794073</v>
       </c>
@@ -1341,19 +1379,19 @@
         <f>I10/I3</f>
         <v>0.92754441689030809</v>
       </c>
-      <c r="K10" s="63">
+      <c r="K10" s="49">
         <f>B10+D10</f>
         <v>29.33</v>
       </c>
-      <c r="L10" s="63">
+      <c r="L10" s="49">
         <f>B10</f>
         <v>11.33</v>
       </c>
-      <c r="M10" s="65">
+      <c r="M10" s="51">
         <f>L10/K10</f>
         <v>0.38629389703375389</v>
       </c>
-      <c r="N10" s="65"/>
+      <c r="N10" s="51"/>
       <c r="Q10" s="12">
         <v>25</v>
       </c>
@@ -1374,7 +1412,7 @@
         <f>U10/U3</f>
         <v>0.97520661157024791</v>
       </c>
-      <c r="W10" s="41">
+      <c r="W10" s="34">
         <f>X10/U10</f>
         <v>0.86748844375963019</v>
       </c>
@@ -1386,30 +1424,30 @@
         <f>X10/X3</f>
         <v>0.9845411303861219</v>
       </c>
-      <c r="Z10" s="63">
+      <c r="Z10" s="49">
         <f>Q10+S10</f>
         <v>68</v>
       </c>
-      <c r="AA10" s="63">
+      <c r="AA10" s="49">
         <f>Q10</f>
         <v>25</v>
       </c>
-      <c r="AB10" s="65">
+      <c r="AB10" s="51">
         <f>AA10/Z10</f>
         <v>0.36764705882352944</v>
       </c>
-      <c r="AC10" s="65"/>
+      <c r="AC10" s="51"/>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.35">
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
-      <c r="H11" s="44"/>
+      <c r="H11" s="8"/>
       <c r="I11" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J11" s="8"/>
-      <c r="K11" s="62"/>
-      <c r="L11" s="62"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="48"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
       <c r="Q11" s="9"/>
@@ -1420,91 +1458,91 @@
       <c r="X11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="Z11" s="62"/>
-      <c r="AA11" s="62"/>
+      <c r="Z11" s="48"/>
+      <c r="AA11" s="48"/>
       <c r="AB11" s="8"/>
       <c r="AC11" s="8"/>
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
+      <c r="C12" s="58"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="58"/>
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
-      <c r="H12" s="44"/>
+      <c r="H12" s="8"/>
       <c r="I12" s="8">
         <f>SUM(D3:E3)</f>
         <v>216.04000000000002</v>
       </c>
       <c r="J12" s="8"/>
-      <c r="K12" s="63" t="s">
+      <c r="K12" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="L12" s="63"/>
+      <c r="L12" s="49"/>
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
-      <c r="Q12" s="34" t="s">
+      <c r="Q12" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="R12" s="34"/>
-      <c r="S12" s="34"/>
-      <c r="T12" s="34"/>
+      <c r="R12" s="58"/>
+      <c r="S12" s="58"/>
+      <c r="T12" s="58"/>
       <c r="U12" s="9"/>
       <c r="X12" s="9">
         <f>SUM(S3:T3)</f>
         <v>187.32</v>
       </c>
-      <c r="Z12" s="63" t="s">
+      <c r="Z12" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="AA12" s="63"/>
+      <c r="AA12" s="49"/>
       <c r="AB12" s="8"/>
       <c r="AC12" s="8"/>
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="B13" s="50"/>
-      <c r="C13" s="50"/>
-      <c r="D13" s="50"/>
-      <c r="E13" s="50"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
-      <c r="H13" s="44"/>
+      <c r="H13" s="8"/>
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
-      <c r="K13" s="61" t="s">
+      <c r="K13" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="L13" s="67" t="s">
+      <c r="L13" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="M13" s="55" t="s">
+      <c r="M13" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="N13" s="68" t="s">
+      <c r="N13" s="54" t="s">
         <v>32</v>
       </c>
       <c r="O13" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="Q13" s="50"/>
-      <c r="R13" s="50"/>
-      <c r="S13" s="50"/>
-      <c r="T13" s="50"/>
+      <c r="Q13" s="32"/>
+      <c r="R13" s="32"/>
+      <c r="S13" s="32"/>
+      <c r="T13" s="32"/>
       <c r="U13" s="9"/>
       <c r="X13" s="9"/>
-      <c r="Z13" s="61" t="s">
+      <c r="Z13" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="AA13" s="67" t="s">
+      <c r="AA13" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="AB13" s="55" t="s">
+      <c r="AB13" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="AC13" s="68" t="s">
+      <c r="AC13" s="54" t="s">
         <v>32</v>
       </c>
       <c r="AD13" s="11" t="s">
@@ -1515,11 +1553,11 @@
       <c r="A14" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="49">
+      <c r="B14" s="7">
         <f>B3-B8</f>
         <v>18.53</v>
       </c>
-      <c r="C14" s="49">
+      <c r="C14" s="7">
         <f>C3-C8</f>
         <v>186.28999999999996</v>
       </c>
@@ -1539,7 +1577,7 @@
         <f>F14/F3</f>
         <v>0.1174095682613769</v>
       </c>
-      <c r="H14" s="38">
+      <c r="H14" s="33">
         <f>I14/F14</f>
         <v>0.32147353077585639</v>
       </c>
@@ -1559,23 +1597,23 @@
         <f>B14+E14</f>
         <v>64.830000000000013</v>
       </c>
-      <c r="M14" s="66">
+      <c r="M14" s="52">
         <f>L14/K14</f>
         <v>0.2147684356986683</v>
       </c>
-      <c r="N14" s="69">
-        <f>K8+K14</f>
+      <c r="N14" s="55">
+        <f t="shared" ref="N14:O16" si="0">K8+K14</f>
         <v>325</v>
       </c>
       <c r="O14" s="14">
-        <f>L8+L14</f>
+        <f t="shared" si="0"/>
         <v>74.970000000000013</v>
       </c>
-      <c r="Q14" s="49">
+      <c r="Q14" s="7">
         <f>Q3-Q8</f>
         <v>26.740000000000002</v>
       </c>
-      <c r="R14" s="49">
+      <c r="R14" s="7">
         <f>R3-R8</f>
         <v>217.94000000000005</v>
       </c>
@@ -1595,7 +1633,7 @@
         <f>U14/U3</f>
         <v>0.27347858752817433</v>
       </c>
-      <c r="W14" s="41">
+      <c r="W14" s="34">
         <f>X14/U14</f>
         <v>0.32780219780219771</v>
       </c>
@@ -1615,16 +1653,16 @@
         <f>Q14+T14</f>
         <v>94.69</v>
       </c>
-      <c r="AB14" s="66">
+      <c r="AB14" s="52">
         <f>AA14/Z14</f>
         <v>0.26013736263736259</v>
       </c>
-      <c r="AC14" s="69">
-        <f>Z8+Z14</f>
+      <c r="AC14" s="55">
+        <f t="shared" ref="AC14:AD16" si="1">Z8+Z14</f>
         <v>376.00000000000006</v>
       </c>
       <c r="AD14" s="14">
-        <f>AA8+AA14</f>
+        <f t="shared" si="1"/>
         <v>100.69</v>
       </c>
     </row>
@@ -1656,7 +1694,7 @@
         <f>F15/F3</f>
         <v>2.5600933488914811E-2</v>
       </c>
-      <c r="H15" s="38">
+      <c r="H15" s="33">
         <f>I15/F15</f>
         <v>0.47158918261926502</v>
       </c>
@@ -1676,16 +1714,16 @@
         <f>B15+E15</f>
         <v>19.790000000000013</v>
       </c>
-      <c r="M15" s="66">
+      <c r="M15" s="52">
         <f>L15/K15</f>
         <v>0.30066848982072347</v>
       </c>
-      <c r="N15" s="69">
-        <f>K9+K15</f>
+      <c r="N15" s="55">
+        <f t="shared" si="0"/>
         <v>132</v>
       </c>
       <c r="O15" s="14">
-        <f>L9+L15</f>
+        <f t="shared" si="0"/>
         <v>40.970000000000013</v>
       </c>
       <c r="Q15" s="7">
@@ -1712,7 +1750,7 @@
         <f>U15/U3</f>
         <v>7.8136739293764121E-2</v>
       </c>
-      <c r="W15" s="41">
+      <c r="W15" s="34">
         <f>X15/U15</f>
         <v>0.49346153846153812</v>
       </c>
@@ -1732,16 +1770,16 @@
         <f>Q15+T15</f>
         <v>32.689999999999991</v>
       </c>
-      <c r="AB15" s="66">
+      <c r="AB15" s="52">
         <f>AA15/Z15</f>
         <v>0.31432692307692284</v>
       </c>
-      <c r="AC15" s="69">
-        <f>Z9+Z15</f>
+      <c r="AC15" s="55">
+        <f t="shared" si="1"/>
         <v>140.00000000000006</v>
       </c>
       <c r="AD15" s="14">
-        <f>AA9+AA15</f>
+        <f t="shared" si="1"/>
         <v>47.689999999999991</v>
       </c>
     </row>
@@ -1773,7 +1811,7 @@
         <f>F16/F3</f>
         <v>0.10022170361726952</v>
       </c>
-      <c r="H16" s="38">
+      <c r="H16" s="33">
         <f>I16/F16</f>
         <v>0.33779640625606411</v>
       </c>
@@ -1793,16 +1831,16 @@
         <f>B16+E16</f>
         <v>58.640000000000015</v>
       </c>
-      <c r="M16" s="66">
+      <c r="M16" s="52">
         <f>L16/K16</f>
         <v>0.22757790972949907</v>
       </c>
-      <c r="N16" s="69">
-        <f>K10+K16</f>
+      <c r="N16" s="55">
+        <f t="shared" si="0"/>
         <v>286.99999999999994</v>
       </c>
       <c r="O16" s="14">
-        <f>L10+L16</f>
+        <f t="shared" si="0"/>
         <v>69.970000000000013</v>
       </c>
       <c r="Q16" s="7">
@@ -1829,7 +1867,7 @@
         <f>U16/U3</f>
         <v>2.4793388429752098E-2</v>
       </c>
-      <c r="W16" s="41">
+      <c r="W16" s="34">
         <f>X16/U16</f>
         <v>0.46424242424242324</v>
       </c>
@@ -1849,50 +1887,50 @@
         <f>Q16+T16</f>
         <v>8.6899999999999906</v>
       </c>
-      <c r="AB16" s="66">
+      <c r="AB16" s="52">
         <f>AA16/Z16</f>
         <v>0.2633333333333327</v>
       </c>
-      <c r="AC16" s="69">
-        <f>Z10+Z16</f>
+      <c r="AC16" s="55">
+        <f t="shared" si="1"/>
         <v>101.00000000000004</v>
       </c>
       <c r="AD16" s="14">
-        <f>AA10+AA16</f>
+        <f t="shared" si="1"/>
         <v>33.689999999999991</v>
       </c>
     </row>
     <row r="17" spans="2:23" x14ac:dyDescent="0.35">
       <c r="U17" s="8"/>
       <c r="V17" s="10"/>
-      <c r="W17" s="45"/>
+      <c r="W17" s="37"/>
     </row>
     <row r="20" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B20" s="11"/>
-      <c r="C20" s="34" t="s">
-        <v>0</v>
-      </c>
-      <c r="D20" s="34"/>
+      <c r="C20" s="58" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="58"/>
       <c r="E20" s="11"/>
       <c r="F20"/>
-      <c r="G20"/>
-      <c r="H20" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="I20" s="34"/>
-      <c r="J20"/>
+      <c r="G20" s="58" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" s="58"/>
+      <c r="I20" s="58"/>
+      <c r="J20" s="58"/>
     </row>
     <row r="21" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B21" s="34" t="s">
+      <c r="B21" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
+      <c r="C21" s="58"/>
+      <c r="D21" s="58"/>
+      <c r="E21" s="58"/>
+      <c r="F21" s="58"/>
+      <c r="G21" s="58"/>
+      <c r="H21" s="58"/>
+      <c r="I21" s="58"/>
       <c r="J21"/>
     </row>
     <row r="22" spans="2:23" x14ac:dyDescent="0.35">
@@ -1903,12 +1941,12 @@
         <v>36</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F22" s="73"/>
+      <c r="F22" s="56"/>
       <c r="G22" s="11" t="s">
         <v>38</v>
       </c>
@@ -1916,41 +1954,41 @@
         <v>36</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J22" s="11" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="23" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B23" s="70">
+      <c r="B23">
         <v>1</v>
       </c>
-      <c r="C23" s="71">
+      <c r="C23" s="9">
         <f>K3</f>
         <v>92.41</v>
       </c>
-      <c r="D23" s="71">
+      <c r="D23" s="9">
         <f>L3</f>
         <v>28.67</v>
       </c>
-      <c r="E23" s="72">
+      <c r="E23" s="18">
         <f>D23/C23</f>
         <v>0.31024780867871443</v>
       </c>
-      <c r="F23" s="73"/>
-      <c r="G23" s="70">
+      <c r="F23" s="56"/>
+      <c r="G23">
         <v>1</v>
       </c>
-      <c r="H23" s="71">
+      <c r="H23" s="9">
         <f>Z3</f>
         <v>90.11</v>
       </c>
-      <c r="I23" s="71">
+      <c r="I23" s="9">
         <f>AA3</f>
         <v>32.74</v>
       </c>
-      <c r="J23" s="72">
+      <c r="J23" s="18">
         <f>I23/H23</f>
         <v>0.36333370325158143</v>
       </c>
@@ -1967,11 +2005,11 @@
         <f>L4</f>
         <v>152.30000000000001</v>
       </c>
-      <c r="E24" s="72">
+      <c r="E24" s="18">
         <f>D24/C24</f>
         <v>6.1446225474967621E-2</v>
       </c>
-      <c r="F24" s="74"/>
+      <c r="F24" s="57"/>
       <c r="G24">
         <v>2</v>
       </c>
@@ -1983,7 +2021,7 @@
         <f>AA4</f>
         <v>129.94999999999999</v>
       </c>
-      <c r="J24" s="72">
+      <c r="J24" s="18">
         <f>I24/H24</f>
         <v>0.10472322284811705</v>
       </c>
@@ -2000,11 +2038,11 @@
         <f>D23+D24</f>
         <v>180.97000000000003</v>
       </c>
-      <c r="E25" s="72">
+      <c r="E25" s="18">
         <f>D25/C25</f>
         <v>7.0388953714507985E-2</v>
       </c>
-      <c r="F25" s="74"/>
+      <c r="F25" s="57"/>
       <c r="G25" t="s">
         <v>39</v>
       </c>
@@ -2016,22 +2054,22 @@
         <f>I23+I24</f>
         <v>162.69</v>
       </c>
-      <c r="J25" s="72">
+      <c r="J25" s="18">
         <f>I25/H25</f>
         <v>0.12223140495867768</v>
       </c>
     </row>
     <row r="26" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B26" s="34" t="s">
+      <c r="B26" s="58" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
+      <c r="C26" s="58"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="58"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58"/>
+      <c r="H26" s="58"/>
+      <c r="I26" s="58"/>
       <c r="J26"/>
     </row>
     <row r="27" spans="2:23" x14ac:dyDescent="0.35">
@@ -2068,11 +2106,11 @@
         <f>L8</f>
         <v>10.14</v>
       </c>
-      <c r="E28" s="72">
+      <c r="E28" s="18">
         <f>D28/C28</f>
         <v>0.43820224719101125</v>
       </c>
-      <c r="F28" s="74"/>
+      <c r="F28" s="57"/>
       <c r="G28">
         <v>1</v>
       </c>
@@ -2084,7 +2122,7 @@
         <f>AA8</f>
         <v>6</v>
       </c>
-      <c r="J28" s="72">
+      <c r="J28" s="18">
         <f>I28/H28</f>
         <v>0.5</v>
       </c>
@@ -2101,11 +2139,11 @@
         <f>L14</f>
         <v>64.830000000000013</v>
       </c>
-      <c r="E29" s="72">
+      <c r="E29" s="18">
         <f>D29/C29</f>
         <v>0.2147684356986683</v>
       </c>
-      <c r="F29" s="74"/>
+      <c r="F29" s="57"/>
       <c r="G29">
         <v>2</v>
       </c>
@@ -2117,7 +2155,7 @@
         <f>AA14</f>
         <v>94.69</v>
       </c>
-      <c r="J29" s="72">
+      <c r="J29" s="18">
         <f>I29/H29</f>
         <v>0.26013736263736259</v>
       </c>
@@ -2134,11 +2172,11 @@
         <f>D28+D29</f>
         <v>74.970000000000013</v>
       </c>
-      <c r="E30" s="72">
+      <c r="E30" s="18">
         <f>D30/C30</f>
         <v>0.23067692307692311</v>
       </c>
-      <c r="F30" s="74"/>
+      <c r="F30" s="57"/>
       <c r="G30" t="s">
         <v>39</v>
       </c>
@@ -2150,22 +2188,22 @@
         <f>I28+I29</f>
         <v>100.69</v>
       </c>
-      <c r="J30" s="72">
+      <c r="J30" s="18">
         <f>I30/H30</f>
         <v>0.26779255319148931</v>
       </c>
     </row>
     <row r="31" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B31" s="34" t="s">
+      <c r="B31" s="58" t="s">
         <v>41</v>
       </c>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="34"/>
-      <c r="F31" s="34"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
+      <c r="C31" s="58"/>
+      <c r="D31" s="58"/>
+      <c r="E31" s="58"/>
+      <c r="F31" s="58"/>
+      <c r="G31" s="58"/>
+      <c r="H31" s="58"/>
+      <c r="I31" s="58"/>
       <c r="J31"/>
     </row>
     <row r="32" spans="2:23" x14ac:dyDescent="0.35">
@@ -2202,11 +2240,11 @@
         <f>L9</f>
         <v>21.18</v>
       </c>
-      <c r="E33" s="72">
+      <c r="E33" s="18">
         <f>D33/C33</f>
         <v>0.32003626473254754</v>
       </c>
-      <c r="F33" s="74"/>
+      <c r="F33" s="57"/>
       <c r="G33">
         <v>1</v>
       </c>
@@ -2218,7 +2256,7 @@
         <f>AA9</f>
         <v>15</v>
       </c>
-      <c r="J33" s="72">
+      <c r="J33" s="18">
         <f>I33/H33</f>
         <v>0.41666666666666669</v>
       </c>
@@ -2235,11 +2273,11 @@
         <f>L15</f>
         <v>19.790000000000013</v>
       </c>
-      <c r="E34" s="72">
+      <c r="E34" s="18">
         <f>D34/C34</f>
         <v>0.30066848982072347</v>
       </c>
-      <c r="F34" s="74"/>
+      <c r="F34" s="57"/>
       <c r="G34">
         <v>2</v>
       </c>
@@ -2251,7 +2289,7 @@
         <f>AA15</f>
         <v>32.689999999999991</v>
       </c>
-      <c r="J34" s="72">
+      <c r="J34" s="18">
         <f>I34/H34</f>
         <v>0.31432692307692284</v>
       </c>
@@ -2268,11 +2306,11 @@
         <f>D33+D34</f>
         <v>40.970000000000013</v>
       </c>
-      <c r="E35" s="72">
+      <c r="E35" s="18">
         <f>D35/C35</f>
         <v>0.31037878787878798</v>
       </c>
-      <c r="F35" s="74"/>
+      <c r="F35" s="57"/>
       <c r="G35" t="s">
         <v>39</v>
       </c>
@@ -2284,22 +2322,22 @@
         <f>I33+I34</f>
         <v>47.689999999999991</v>
       </c>
-      <c r="J35" s="72">
+      <c r="J35" s="18">
         <f>I35/H35</f>
         <v>0.34064285714285691</v>
       </c>
     </row>
     <row r="36" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B36" s="34" t="s">
+      <c r="B36" s="58" t="s">
         <v>42</v>
       </c>
-      <c r="C36" s="34"/>
-      <c r="D36" s="34"/>
-      <c r="E36" s="34"/>
-      <c r="F36" s="34"/>
-      <c r="G36" s="34"/>
-      <c r="H36" s="34"/>
-      <c r="I36" s="34"/>
+      <c r="C36" s="58"/>
+      <c r="D36" s="58"/>
+      <c r="E36" s="58"/>
+      <c r="F36" s="58"/>
+      <c r="G36" s="58"/>
+      <c r="H36" s="58"/>
+      <c r="I36" s="58"/>
       <c r="J36"/>
     </row>
     <row r="37" spans="2:29" x14ac:dyDescent="0.35">
@@ -2336,11 +2374,11 @@
         <f>L10</f>
         <v>11.33</v>
       </c>
-      <c r="E38" s="72">
+      <c r="E38" s="18">
         <f>D38/C38</f>
         <v>0.38629389703375389</v>
       </c>
-      <c r="F38" s="74"/>
+      <c r="F38" s="57"/>
       <c r="G38">
         <v>1</v>
       </c>
@@ -2352,7 +2390,7 @@
         <f>AA10</f>
         <v>25</v>
       </c>
-      <c r="J38" s="72">
+      <c r="J38" s="18">
         <f>I38/H38</f>
         <v>0.36764705882352944</v>
       </c>
@@ -2369,11 +2407,11 @@
         <f>L16</f>
         <v>58.640000000000015</v>
       </c>
-      <c r="E39" s="72">
+      <c r="E39" s="18">
         <f>D39/C39</f>
         <v>0.22757790972949907</v>
       </c>
-      <c r="F39" s="74"/>
+      <c r="F39" s="57"/>
       <c r="G39">
         <v>2</v>
       </c>
@@ -2385,7 +2423,7 @@
         <f>AA16</f>
         <v>8.6899999999999906</v>
       </c>
-      <c r="J39" s="72">
+      <c r="J39" s="18">
         <f>I39/H39</f>
         <v>0.2633333333333327</v>
       </c>
@@ -2402,11 +2440,11 @@
         <f>D38+D39</f>
         <v>69.970000000000013</v>
       </c>
-      <c r="E40" s="72">
+      <c r="E40" s="18">
         <f>D40/C40</f>
         <v>0.2437979094076656</v>
       </c>
-      <c r="F40" s="74"/>
+      <c r="F40" s="57"/>
       <c r="G40" t="s">
         <v>39</v>
       </c>
@@ -2418,7 +2456,7 @@
         <f>I38+I39</f>
         <v>33.689999999999991</v>
       </c>
-      <c r="J40" s="72">
+      <c r="J40" s="18">
         <f>I40/H40</f>
         <v>0.33356435643564331</v>
       </c>
@@ -2426,7 +2464,7 @@
     <row r="41" spans="2:29" x14ac:dyDescent="0.35">
       <c r="F41"/>
       <c r="G41"/>
-      <c r="H41" s="37"/>
+      <c r="H41"/>
       <c r="I41"/>
       <c r="J41"/>
       <c r="U41" s="3"/>
@@ -2434,18 +2472,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B26:I26"/>
-    <mergeCell ref="B31:I31"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="Q1:T1"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="Q6:T6"/>
     <mergeCell ref="Q12:T12"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B26:I26"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="G20:J20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2461,52 +2499,52 @@
     <col min="4" max="4" width="8.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.77734375" customWidth="1"/>
-    <col min="8" max="8" width="8.5546875" style="37" customWidth="1"/>
+    <col min="8" max="8" width="8.5546875" customWidth="1"/>
     <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.33203125" customWidth="1"/>
-    <col min="11" max="11" width="33.21875" style="61" customWidth="1"/>
-    <col min="12" max="12" width="17" style="61" customWidth="1"/>
+    <col min="11" max="11" width="33.21875" style="47" customWidth="1"/>
+    <col min="12" max="12" width="17" style="47" customWidth="1"/>
     <col min="13" max="13" width="8.33203125" style="1" customWidth="1"/>
     <col min="14" max="14" width="16.6640625" style="1" customWidth="1"/>
     <col min="15" max="15" width="20.33203125" customWidth="1"/>
-    <col min="16" max="16" width="7.21875" style="52" customWidth="1"/>
+    <col min="16" max="16" width="7.21875" style="40" customWidth="1"/>
     <col min="17" max="17" width="8.77734375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="19" max="20" width="8.77734375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="9.21875" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.77734375" style="37"/>
+    <col min="23" max="23" width="8.77734375"/>
     <col min="25" max="25" width="9.109375" customWidth="1"/>
-    <col min="26" max="26" width="33.21875" style="61" customWidth="1"/>
-    <col min="27" max="27" width="17" style="61" customWidth="1"/>
+    <col min="26" max="26" width="33.21875" style="47" customWidth="1"/>
+    <col min="27" max="27" width="17" style="47" customWidth="1"/>
     <col min="28" max="28" width="8.33203125" style="1" customWidth="1"/>
     <col min="29" max="29" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="52" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="53" t="s">
+    <row r="1" spans="1:30" s="40" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="Q1" s="53" t="s">
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="Q1" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="53"/>
-      <c r="S1" s="53"/>
-      <c r="T1" s="53"/>
-      <c r="Z1" s="54"/>
-      <c r="AA1" s="54"/>
-      <c r="AB1" s="56"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="59"/>
+      <c r="Z1" s="41"/>
+      <c r="AA1" s="41"/>
+      <c r="AB1" s="43"/>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
@@ -2527,16 +2565,16 @@
       <c r="I2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="60" t="s">
+      <c r="K2" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="67" t="s">
+      <c r="L2" s="53" t="s">
         <v>28</v>
       </c>
       <c r="M2" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="N2" s="57"/>
+      <c r="N2" s="20"/>
       <c r="Q2" s="2" t="s">
         <v>2</v>
       </c>
@@ -2557,10 +2595,10 @@
         <v>16</v>
       </c>
       <c r="Y2" s="3"/>
-      <c r="Z2" s="60" t="s">
+      <c r="Z2" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="AA2" s="67" t="s">
+      <c r="AA2" s="53" t="s">
         <v>28</v>
       </c>
       <c r="AB2" s="24" t="s">
@@ -2588,26 +2626,26 @@
         <v>4783</v>
       </c>
       <c r="G3" s="13"/>
-      <c r="H3" s="36"/>
+      <c r="H3" s="13"/>
       <c r="I3" s="26">
         <f>SUM(B3:C3)</f>
         <v>4088</v>
       </c>
       <c r="J3" s="13"/>
-      <c r="K3" s="60">
+      <c r="K3" s="46">
         <f>B3+D3</f>
         <v>50</v>
       </c>
-      <c r="L3" s="60">
+      <c r="L3" s="46">
         <f>B3</f>
         <v>25</v>
       </c>
-      <c r="M3" s="65">
+      <c r="M3" s="51">
         <f>L3/K3</f>
         <v>0.5</v>
       </c>
       <c r="N3" s="24"/>
-      <c r="P3" s="52"/>
+      <c r="P3" s="40"/>
       <c r="Q3" s="11">
         <v>201</v>
       </c>
@@ -2625,20 +2663,19 @@
         <v>4552</v>
       </c>
       <c r="V3" s="13"/>
-      <c r="W3" s="39"/>
       <c r="X3" s="3">
         <f>SUM(Q3:R3)</f>
         <v>3707</v>
       </c>
-      <c r="Z3" s="60">
+      <c r="Z3" s="46">
         <f>Q3+S3</f>
         <v>372</v>
       </c>
-      <c r="AA3" s="60">
+      <c r="AA3" s="46">
         <f>Q3</f>
         <v>201</v>
       </c>
-      <c r="AB3" s="65">
+      <c r="AB3" s="51">
         <f>AA3/Z3</f>
         <v>0.54032258064516125</v>
       </c>
@@ -2646,14 +2683,14 @@
     <row r="4" spans="1:30" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
-      <c r="H4" s="36"/>
+      <c r="H4" s="13"/>
       <c r="I4" s="26"/>
       <c r="J4" s="13"/>
-      <c r="K4" s="60">
+      <c r="K4" s="46">
         <f>C3+E3</f>
         <v>4733</v>
       </c>
-      <c r="L4" s="60">
+      <c r="L4" s="46">
         <f>E3</f>
         <v>670</v>
       </c>
@@ -2661,17 +2698,16 @@
         <f>L4/K4</f>
         <v>0.14155926473695329</v>
       </c>
-      <c r="N4" s="65"/>
-      <c r="P4" s="52"/>
+      <c r="N4" s="51"/>
+      <c r="P4" s="40"/>
       <c r="U4" s="3"/>
       <c r="V4" s="13"/>
-      <c r="W4" s="39"/>
       <c r="X4" s="3"/>
-      <c r="Z4" s="60">
+      <c r="Z4" s="46">
         <f>R3+T3</f>
         <v>4180</v>
       </c>
-      <c r="AA4" s="60">
+      <c r="AA4" s="46">
         <f>T3</f>
         <v>674</v>
       </c>
@@ -2683,33 +2719,32 @@
     <row r="5" spans="1:30" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
-      <c r="H5" s="36"/>
+      <c r="H5" s="13"/>
       <c r="I5" s="26"/>
       <c r="J5" s="13"/>
       <c r="N5" s="24"/>
-      <c r="P5" s="52"/>
+      <c r="P5" s="40"/>
       <c r="U5" s="3"/>
       <c r="V5" s="13"/>
-      <c r="W5" s="39"/>
       <c r="X5" s="9"/>
-      <c r="Z5" s="60"/>
-      <c r="AA5" s="60"/>
+      <c r="Z5" s="46"/>
+      <c r="AA5" s="46"/>
       <c r="AB5" s="24"/>
     </row>
     <row r="6" spans="1:30" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
       <c r="F6" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="36" t="s">
+      <c r="H6" s="13" t="s">
         <v>18</v>
       </c>
       <c r="I6" s="3" t="s">
@@ -2718,26 +2753,26 @@
       <c r="J6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K6" s="67" t="s">
+      <c r="K6" s="53" t="s">
         <v>27</v>
       </c>
       <c r="L6" s="3"/>
-      <c r="M6" s="58"/>
-      <c r="N6" s="58"/>
-      <c r="P6" s="52"/>
-      <c r="Q6" s="33" t="s">
+      <c r="M6" s="44"/>
+      <c r="N6" s="44"/>
+      <c r="P6" s="40"/>
+      <c r="Q6" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="R6" s="33"/>
-      <c r="S6" s="33"/>
-      <c r="T6" s="33"/>
+      <c r="R6" s="60"/>
+      <c r="S6" s="60"/>
+      <c r="T6" s="60"/>
       <c r="U6" s="3" t="s">
         <v>24</v>
       </c>
       <c r="V6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="W6" s="36" t="s">
+      <c r="W6" s="13" t="s">
         <v>18</v>
       </c>
       <c r="X6" s="3" t="s">
@@ -2746,11 +2781,11 @@
       <c r="Y6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="Z6" s="67" t="s">
+      <c r="Z6" s="53" t="s">
         <v>27</v>
       </c>
       <c r="AA6" s="3"/>
-      <c r="AB6" s="58"/>
+      <c r="AB6" s="44"/>
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
@@ -2760,24 +2795,24 @@
       <c r="G7" s="13"/>
       <c r="I7" s="13"/>
       <c r="J7" s="13"/>
-      <c r="K7" s="61" t="s">
+      <c r="K7" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="L7" s="67" t="s">
+      <c r="L7" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="M7" s="55" t="s">
+      <c r="M7" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="N7" s="55"/>
+      <c r="N7" s="42"/>
       <c r="Y7" s="13"/>
-      <c r="Z7" s="61" t="s">
+      <c r="Z7" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="AA7" s="67" t="s">
+      <c r="AA7" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="AB7" s="55" t="s">
+      <c r="AB7" s="42" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2805,7 +2840,7 @@
         <f>F8/F3</f>
         <v>0.56596278486305662</v>
       </c>
-      <c r="H8" s="38">
+      <c r="H8" s="33">
         <f>I8/F8</f>
         <v>0.90690801625415585</v>
       </c>
@@ -2817,19 +2852,19 @@
         <f>I8/I3</f>
         <v>0.60053816046966735</v>
       </c>
-      <c r="K8" s="63">
+      <c r="K8" s="49">
         <f>B8+D8</f>
         <v>4</v>
       </c>
-      <c r="L8" s="63">
+      <c r="L8" s="49">
         <f>B8</f>
         <v>1</v>
       </c>
-      <c r="M8" s="65">
+      <c r="M8" s="51">
         <f>L8/K8</f>
         <v>0.25</v>
       </c>
-      <c r="N8" s="65"/>
+      <c r="N8" s="51"/>
       <c r="Q8" s="12">
         <v>33</v>
       </c>
@@ -2850,7 +2885,7 @@
         <f>U8/U3</f>
         <v>0.39806678383128297</v>
       </c>
-      <c r="W8" s="40">
+      <c r="W8" s="18">
         <f>X8/U8</f>
         <v>0.91280353200883002</v>
       </c>
@@ -2862,15 +2897,15 @@
         <f>X8/X3</f>
         <v>0.44618289722147286</v>
       </c>
-      <c r="Z8" s="63">
+      <c r="Z8" s="49">
         <f>Q8+S8</f>
         <v>41</v>
       </c>
-      <c r="AA8" s="63">
+      <c r="AA8" s="49">
         <f>Q8</f>
         <v>33</v>
       </c>
-      <c r="AB8" s="65">
+      <c r="AB8" s="51">
         <f>AA8/Z8</f>
         <v>0.80487804878048785</v>
       </c>
@@ -2899,7 +2934,7 @@
         <f>F9/F3</f>
         <v>0.84653982855948151</v>
       </c>
-      <c r="H9" s="38">
+      <c r="H9" s="33">
         <f>I9/F9</f>
         <v>0.87873549024450481</v>
       </c>
@@ -2911,19 +2946,19 @@
         <f>I9/I3</f>
         <v>0.87035225048923681</v>
       </c>
-      <c r="K9" s="63">
+      <c r="K9" s="49">
         <f>B9+D9</f>
         <v>10</v>
       </c>
-      <c r="L9" s="63">
+      <c r="L9" s="49">
         <f>B9</f>
         <v>5</v>
       </c>
-      <c r="M9" s="65">
+      <c r="M9" s="51">
         <f>L9/K9</f>
         <v>0.5</v>
       </c>
-      <c r="N9" s="65"/>
+      <c r="N9" s="51"/>
       <c r="Q9" s="12">
         <v>52</v>
       </c>
@@ -2944,7 +2979,7 @@
         <f>U9/U3</f>
         <v>0.60896309314586994</v>
       </c>
-      <c r="W9" s="40">
+      <c r="W9" s="18">
         <f>X9/U9</f>
         <v>0.88997113997113997</v>
       </c>
@@ -2956,15 +2991,15 @@
         <f>X9/X3</f>
         <v>0.66549770704073374</v>
       </c>
-      <c r="Z9" s="63">
+      <c r="Z9" s="49">
         <f>Q9+S9</f>
         <v>74</v>
       </c>
-      <c r="AA9" s="63">
+      <c r="AA9" s="49">
         <f>Q9</f>
         <v>52</v>
       </c>
-      <c r="AB9" s="65">
+      <c r="AB9" s="51">
         <f>AA9/Z9</f>
         <v>0.70270270270270274</v>
       </c>
@@ -2993,7 +3028,7 @@
         <f>F10/F3</f>
         <v>0.98201965293748694</v>
       </c>
-      <c r="H10" s="38">
+      <c r="H10" s="33">
         <f>I10/F10</f>
         <v>0.85884607196082607</v>
       </c>
@@ -3005,19 +3040,19 @@
         <f>I10/I3</f>
         <v>0.98679060665362039</v>
       </c>
-      <c r="K10" s="63">
+      <c r="K10" s="49">
         <f>B10+D10</f>
         <v>27</v>
       </c>
-      <c r="L10" s="63">
+      <c r="L10" s="49">
         <f>B10</f>
         <v>15</v>
       </c>
-      <c r="M10" s="65">
+      <c r="M10" s="51">
         <f>L10/K10</f>
         <v>0.55555555555555558</v>
       </c>
-      <c r="N10" s="65"/>
+      <c r="N10" s="51"/>
       <c r="Q10" s="12">
         <v>92</v>
       </c>
@@ -3038,7 +3073,7 @@
         <f>U10/U3</f>
         <v>0.7752636203866432</v>
       </c>
-      <c r="W10" s="40">
+      <c r="W10" s="18">
         <f>X10/U10</f>
         <v>0.8642674978747521</v>
       </c>
@@ -3050,15 +3085,15 @@
         <f>X10/X3</f>
         <v>0.82276773671432424</v>
       </c>
-      <c r="Z10" s="63">
+      <c r="Z10" s="49">
         <f>Q10+S10</f>
         <v>136</v>
       </c>
-      <c r="AA10" s="63">
+      <c r="AA10" s="49">
         <f>Q10</f>
         <v>92</v>
       </c>
-      <c r="AB10" s="65">
+      <c r="AB10" s="51">
         <f>AA10/Z10</f>
         <v>0.67647058823529416</v>
       </c>
@@ -3070,11 +3105,11 @@
       <c r="E11" s="9"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
-      <c r="H11" s="36"/>
+      <c r="H11" s="13"/>
       <c r="I11" s="13"/>
       <c r="J11" s="13"/>
-      <c r="K11" s="62"/>
-      <c r="L11" s="62"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="48"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
       <c r="Q11" s="19"/>
@@ -3082,44 +3117,44 @@
       <c r="S11" s="9"/>
       <c r="T11" s="9"/>
       <c r="U11" s="13"/>
-      <c r="Z11" s="62"/>
-      <c r="AA11" s="62"/>
+      <c r="Z11" s="48"/>
+      <c r="AA11" s="48"/>
       <c r="AB11" s="8"/>
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
+      <c r="C12" s="58"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="58"/>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
-      <c r="H12" s="36"/>
+      <c r="H12" s="13"/>
       <c r="I12" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J12" s="13"/>
-      <c r="K12" s="63" t="s">
+      <c r="K12" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="L12" s="63"/>
+      <c r="L12" s="49"/>
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
-      <c r="Q12" s="34" t="s">
+      <c r="Q12" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="R12" s="34"/>
-      <c r="S12" s="34"/>
-      <c r="T12" s="34"/>
+      <c r="R12" s="58"/>
+      <c r="S12" s="58"/>
+      <c r="T12" s="58"/>
       <c r="U12" s="13"/>
       <c r="X12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="Z12" s="63" t="s">
+      <c r="Z12" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="AA12" s="63"/>
+      <c r="AA12" s="49"/>
       <c r="AB12" s="8"/>
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.35">
@@ -3132,21 +3167,21 @@
       <c r="E13" s="9"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
-      <c r="H13" s="36"/>
+      <c r="H13" s="13"/>
       <c r="I13" s="13">
         <f>SUM(D3:E3)</f>
         <v>695</v>
       </c>
-      <c r="K13" s="61" t="s">
+      <c r="K13" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="L13" s="67" t="s">
+      <c r="L13" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="M13" s="55" t="s">
+      <c r="M13" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="N13" s="68" t="s">
+      <c r="N13" s="54" t="s">
         <v>32</v>
       </c>
       <c r="O13" s="11" t="s">
@@ -3162,16 +3197,16 @@
         <f>SUM(S3:T3)</f>
         <v>845</v>
       </c>
-      <c r="Z13" s="61" t="s">
+      <c r="Z13" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="AA13" s="67" t="s">
+      <c r="AA13" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="AB13" s="55" t="s">
+      <c r="AB13" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="AC13" s="68" t="s">
+      <c r="AC13" s="54" t="s">
         <v>32</v>
       </c>
       <c r="AD13" s="11" t="s">
@@ -3182,11 +3217,11 @@
       <c r="A14" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="49">
+      <c r="B14" s="7">
         <f>B3-B8</f>
         <v>24</v>
       </c>
-      <c r="C14" s="49">
+      <c r="C14" s="7">
         <f>C3-C8</f>
         <v>1609</v>
       </c>
@@ -3206,7 +3241,7 @@
         <f>F14/F3</f>
         <v>0.43403721513694332</v>
       </c>
-      <c r="H14" s="38">
+      <c r="H14" s="33">
         <f>I14/F14</f>
         <v>0.21339113680154143</v>
       </c>
@@ -3226,23 +3261,23 @@
         <f>B14+E14</f>
         <v>445</v>
       </c>
-      <c r="M14" s="66">
+      <c r="M14" s="52">
         <f>L14/K14</f>
         <v>0.21435452793834298</v>
       </c>
-      <c r="N14" s="69">
-        <f>K8+K14</f>
+      <c r="N14" s="55">
+        <f t="shared" ref="N14:O16" si="0">K8+K14</f>
         <v>2080</v>
       </c>
       <c r="O14" s="14">
-        <f>L8+L14</f>
+        <f t="shared" si="0"/>
         <v>446</v>
       </c>
-      <c r="Q14" s="49">
+      <c r="Q14" s="7">
         <f>Q3-Q8</f>
         <v>168</v>
       </c>
-      <c r="R14" s="49">
+      <c r="R14" s="7">
         <f>R3-R8</f>
         <v>1885</v>
       </c>
@@ -3262,7 +3297,7 @@
         <f>U14/U3</f>
         <v>0.60193321616871709</v>
       </c>
-      <c r="W14" s="41">
+      <c r="W14" s="34">
         <f>X14/U14</f>
         <v>0.25072992700729929</v>
       </c>
@@ -3282,16 +3317,16 @@
         <f>Q14+T14</f>
         <v>692</v>
       </c>
-      <c r="AB14" s="66">
+      <c r="AB14" s="52">
         <f>AA14/Z14</f>
         <v>0.25255474452554744</v>
       </c>
-      <c r="AC14" s="69">
-        <f>Z8+Z14</f>
+      <c r="AC14" s="55">
+        <f t="shared" ref="AC14:AD16" si="1">Z8+Z14</f>
         <v>2781</v>
       </c>
       <c r="AD14" s="14">
-        <f>AA8+AA14</f>
+        <f t="shared" si="1"/>
         <v>725</v>
       </c>
     </row>
@@ -3323,7 +3358,7 @@
         <f>F15/F3</f>
         <v>0.15346017144051852</v>
       </c>
-      <c r="H15" s="38">
+      <c r="H15" s="33">
         <f>I15/F15</f>
         <v>0.27792915531335149</v>
       </c>
@@ -3343,16 +3378,16 @@
         <f>B15+E15</f>
         <v>204</v>
       </c>
-      <c r="M15" s="66">
+      <c r="M15" s="52">
         <f>L15/K15</f>
         <v>0.27792915531335149</v>
       </c>
-      <c r="N15" s="69">
-        <f>K9+K15</f>
+      <c r="N15" s="55">
+        <f t="shared" si="0"/>
         <v>744</v>
       </c>
       <c r="O15" s="14">
-        <f>L9+L15</f>
+        <f t="shared" si="0"/>
         <v>209</v>
       </c>
       <c r="Q15" s="7">
@@ -3379,7 +3414,7 @@
         <f>U15/U3</f>
         <v>0.39103690685413006</v>
       </c>
-      <c r="W15" s="41">
+      <c r="W15" s="34">
         <f>X15/U15</f>
         <v>0.30337078651685395</v>
       </c>
@@ -3399,16 +3434,16 @@
         <f>Q15+T15</f>
         <v>540</v>
       </c>
-      <c r="AB15" s="66">
+      <c r="AB15" s="52">
         <f>AA15/Z15</f>
         <v>0.30337078651685395</v>
       </c>
-      <c r="AC15" s="69">
-        <f>Z9+Z15</f>
+      <c r="AC15" s="55">
+        <f t="shared" si="1"/>
         <v>1854</v>
       </c>
       <c r="AD15" s="14">
-        <f>AA9+AA15</f>
+        <f t="shared" si="1"/>
         <v>592</v>
       </c>
     </row>
@@ -3440,7 +3475,7 @@
         <f>F16/F3</f>
         <v>1.7980347062513068E-2</v>
       </c>
-      <c r="H16" s="38">
+      <c r="H16" s="33">
         <f>I16/F16</f>
         <v>0.37209302325581395</v>
       </c>
@@ -3460,16 +3495,16 @@
         <f>B16+E16</f>
         <v>29</v>
       </c>
-      <c r="M16" s="66">
+      <c r="M16" s="52">
         <f>L16/K16</f>
         <v>0.33720930232558138</v>
       </c>
-      <c r="N16" s="69">
-        <f>K10+K16</f>
+      <c r="N16" s="55">
+        <f t="shared" si="0"/>
         <v>113</v>
       </c>
       <c r="O16" s="14">
-        <f>L10+L16</f>
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="Q16" s="7">
@@ -3496,7 +3531,7 @@
         <f>U16/U3</f>
         <v>0.22473637961335677</v>
       </c>
-      <c r="W16" s="41">
+      <c r="W16" s="34">
         <f>X16/U16</f>
         <v>0.35777126099706746</v>
       </c>
@@ -3516,16 +3551,16 @@
         <f>Q16+T16</f>
         <v>348</v>
       </c>
-      <c r="AB16" s="66">
+      <c r="AB16" s="52">
         <f>AA16/Z16</f>
         <v>0.34017595307917886</v>
       </c>
-      <c r="AC16" s="69">
-        <f>Z10+Z16</f>
+      <c r="AC16" s="55">
+        <f t="shared" si="1"/>
         <v>1159</v>
       </c>
       <c r="AD16" s="14">
-        <f>AA10+AA16</f>
+        <f t="shared" si="1"/>
         <v>440</v>
       </c>
     </row>
@@ -3536,35 +3571,37 @@
       <c r="E17" s="9"/>
       <c r="F17" s="13"/>
       <c r="G17" s="16"/>
-      <c r="H17" s="38"/>
+      <c r="H17" s="33"/>
       <c r="I17" s="13"/>
       <c r="J17" s="16"/>
     </row>
     <row r="20" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B20" s="11"/>
-      <c r="C20" s="34" t="s">
-        <v>0</v>
-      </c>
-      <c r="D20" s="34"/>
-      <c r="E20" s="11"/>
-      <c r="H20" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="I20" s="34"/>
+      <c r="B20" s="58" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="58"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="58"/>
+      <c r="G20" s="58" t="s">
+        <v>47</v>
+      </c>
+      <c r="H20" s="58"/>
+      <c r="I20" s="58"/>
+      <c r="J20" s="58"/>
       <c r="U20"/>
       <c r="AC20" s="1"/>
     </row>
     <row r="21" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B21" s="34" t="s">
+      <c r="B21" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
+      <c r="C21" s="58"/>
+      <c r="D21" s="58"/>
+      <c r="E21" s="58"/>
+      <c r="F21" s="58"/>
+      <c r="G21" s="58"/>
+      <c r="H21" s="58"/>
+      <c r="I21" s="58"/>
       <c r="U21"/>
       <c r="AC21" s="1"/>
     </row>
@@ -3576,12 +3613,12 @@
         <v>36</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F22" s="73"/>
+      <c r="F22" s="56"/>
       <c r="G22" s="11" t="s">
         <v>38</v>
       </c>
@@ -3589,7 +3626,7 @@
         <v>36</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J22" s="11" t="s">
         <v>26</v>
@@ -3598,34 +3635,34 @@
       <c r="AC22" s="1"/>
     </row>
     <row r="23" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B23" s="70">
+      <c r="B23">
         <v>1</v>
       </c>
-      <c r="C23" s="71">
+      <c r="C23" s="9">
         <f>K3</f>
         <v>50</v>
       </c>
-      <c r="D23" s="71">
+      <c r="D23" s="9">
         <f>L3</f>
         <v>25</v>
       </c>
-      <c r="E23" s="72">
+      <c r="E23" s="18">
         <f>D23/C23</f>
         <v>0.5</v>
       </c>
-      <c r="F23" s="73"/>
-      <c r="G23" s="70">
+      <c r="F23" s="56"/>
+      <c r="G23">
         <v>1</v>
       </c>
-      <c r="H23" s="71">
+      <c r="H23" s="9">
         <f>Z3</f>
         <v>372</v>
       </c>
-      <c r="I23" s="71">
+      <c r="I23" s="9">
         <f>AA3</f>
         <v>201</v>
       </c>
-      <c r="J23" s="72">
+      <c r="J23" s="18">
         <f>I23/H23</f>
         <v>0.54032258064516125</v>
       </c>
@@ -3644,11 +3681,11 @@
         <f>L4</f>
         <v>670</v>
       </c>
-      <c r="E24" s="72">
+      <c r="E24" s="18">
         <f>D24/C24</f>
         <v>0.14155926473695329</v>
       </c>
-      <c r="F24" s="74"/>
+      <c r="F24" s="57"/>
       <c r="G24">
         <v>2</v>
       </c>
@@ -3660,7 +3697,7 @@
         <f>AA4</f>
         <v>674</v>
       </c>
-      <c r="J24" s="72">
+      <c r="J24" s="18">
         <f>I24/H24</f>
         <v>0.16124401913875597</v>
       </c>
@@ -3679,11 +3716,11 @@
         <f>D23+D24</f>
         <v>695</v>
       </c>
-      <c r="E25" s="72">
+      <c r="E25" s="18">
         <f>D25/C25</f>
         <v>0.14530629312147189</v>
       </c>
-      <c r="F25" s="74"/>
+      <c r="F25" s="57"/>
       <c r="G25" t="s">
         <v>39</v>
       </c>
@@ -3695,7 +3732,7 @@
         <f>I23+I24</f>
         <v>875</v>
       </c>
-      <c r="J25" s="72">
+      <c r="J25" s="18">
         <f>I25/H25</f>
         <v>0.19222319859402459</v>
       </c>
@@ -3703,16 +3740,16 @@
       <c r="AC25" s="1"/>
     </row>
     <row r="26" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="61" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="32"/>
+      <c r="C26" s="61"/>
+      <c r="D26" s="61"/>
+      <c r="E26" s="61"/>
+      <c r="F26" s="61"/>
+      <c r="G26" s="61"/>
+      <c r="H26" s="61"/>
+      <c r="I26" s="61"/>
       <c r="U26"/>
       <c r="AC26" s="1"/>
     </row>
@@ -3750,11 +3787,11 @@
         <f>L8</f>
         <v>1</v>
       </c>
-      <c r="E28" s="72">
+      <c r="E28" s="18">
         <f>D28/C28</f>
         <v>0.25</v>
       </c>
-      <c r="F28" s="74"/>
+      <c r="F28" s="57"/>
       <c r="G28">
         <v>1</v>
       </c>
@@ -3766,7 +3803,7 @@
         <f>AA8</f>
         <v>33</v>
       </c>
-      <c r="J28" s="72">
+      <c r="J28" s="18">
         <f>I28/H28</f>
         <v>0.80487804878048785</v>
       </c>
@@ -3785,11 +3822,11 @@
         <f>L14</f>
         <v>445</v>
       </c>
-      <c r="E29" s="72">
+      <c r="E29" s="18">
         <f>D29/C29</f>
         <v>0.21435452793834298</v>
       </c>
-      <c r="F29" s="74"/>
+      <c r="F29" s="57"/>
       <c r="G29">
         <v>2</v>
       </c>
@@ -3801,7 +3838,7 @@
         <f>AA14</f>
         <v>692</v>
       </c>
-      <c r="J29" s="72">
+      <c r="J29" s="18">
         <f>I29/H29</f>
         <v>0.25255474452554744</v>
       </c>
@@ -3820,11 +3857,11 @@
         <f>D28+D29</f>
         <v>446</v>
       </c>
-      <c r="E30" s="72">
+      <c r="E30" s="18">
         <f>D30/C30</f>
         <v>0.21442307692307691</v>
       </c>
-      <c r="F30" s="74"/>
+      <c r="F30" s="57"/>
       <c r="G30" t="s">
         <v>39</v>
       </c>
@@ -3836,7 +3873,7 @@
         <f>I28+I29</f>
         <v>725</v>
       </c>
-      <c r="J30" s="72">
+      <c r="J30" s="18">
         <f>I30/H30</f>
         <v>0.26069759079467819</v>
       </c>
@@ -3844,16 +3881,16 @@
       <c r="AC30" s="1"/>
     </row>
     <row r="31" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="32"/>
+      <c r="C31" s="61"/>
+      <c r="D31" s="61"/>
+      <c r="E31" s="61"/>
+      <c r="F31" s="61"/>
+      <c r="G31" s="61"/>
+      <c r="H31" s="61"/>
+      <c r="I31" s="61"/>
       <c r="U31"/>
       <c r="AC31" s="1"/>
     </row>
@@ -3891,11 +3928,11 @@
         <f>L9</f>
         <v>5</v>
       </c>
-      <c r="E33" s="72">
+      <c r="E33" s="18">
         <f>D33/C33</f>
         <v>0.5</v>
       </c>
-      <c r="F33" s="74"/>
+      <c r="F33" s="57"/>
       <c r="G33">
         <v>1</v>
       </c>
@@ -3907,7 +3944,7 @@
         <f>AA9</f>
         <v>52</v>
       </c>
-      <c r="J33" s="72">
+      <c r="J33" s="18">
         <f>I33/H33</f>
         <v>0.70270270270270274</v>
       </c>
@@ -3926,11 +3963,11 @@
         <f>L15</f>
         <v>204</v>
       </c>
-      <c r="E34" s="72">
+      <c r="E34" s="18">
         <f>D34/C34</f>
         <v>0.27792915531335149</v>
       </c>
-      <c r="F34" s="74"/>
+      <c r="F34" s="57"/>
       <c r="G34">
         <v>2</v>
       </c>
@@ -3942,7 +3979,7 @@
         <f>AA15</f>
         <v>540</v>
       </c>
-      <c r="J34" s="72">
+      <c r="J34" s="18">
         <f>I34/H34</f>
         <v>0.30337078651685395</v>
       </c>
@@ -3961,11 +3998,11 @@
         <f>D33+D34</f>
         <v>209</v>
       </c>
-      <c r="E35" s="72">
+      <c r="E35" s="18">
         <f>D35/C35</f>
         <v>0.28091397849462363</v>
       </c>
-      <c r="F35" s="74"/>
+      <c r="F35" s="57"/>
       <c r="G35" t="s">
         <v>39</v>
       </c>
@@ -3977,7 +4014,7 @@
         <f>I33+I34</f>
         <v>592</v>
       </c>
-      <c r="J35" s="72">
+      <c r="J35" s="18">
         <f>I35/H35</f>
         <v>0.31930960086299892</v>
       </c>
@@ -3985,16 +4022,16 @@
       <c r="AC35" s="1"/>
     </row>
     <row r="36" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B36" s="32" t="s">
+      <c r="B36" s="61" t="s">
         <v>42</v>
       </c>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-      <c r="H36" s="32"/>
-      <c r="I36" s="32"/>
+      <c r="C36" s="61"/>
+      <c r="D36" s="61"/>
+      <c r="E36" s="61"/>
+      <c r="F36" s="61"/>
+      <c r="G36" s="61"/>
+      <c r="H36" s="61"/>
+      <c r="I36" s="61"/>
       <c r="U36"/>
       <c r="AC36" s="1"/>
     </row>
@@ -4032,11 +4069,11 @@
         <f>L10</f>
         <v>15</v>
       </c>
-      <c r="E38" s="72">
+      <c r="E38" s="18">
         <f>D38/C38</f>
         <v>0.55555555555555558</v>
       </c>
-      <c r="F38" s="74"/>
+      <c r="F38" s="57"/>
       <c r="G38">
         <v>1</v>
       </c>
@@ -4048,7 +4085,7 @@
         <f>AA10</f>
         <v>92</v>
       </c>
-      <c r="J38" s="72">
+      <c r="J38" s="18">
         <f>I38/H38</f>
         <v>0.67647058823529416</v>
       </c>
@@ -4067,11 +4104,11 @@
         <f>L16</f>
         <v>29</v>
       </c>
-      <c r="E39" s="72">
+      <c r="E39" s="18">
         <f>D39/C39</f>
         <v>0.33720930232558138</v>
       </c>
-      <c r="F39" s="74"/>
+      <c r="F39" s="57"/>
       <c r="G39">
         <v>2</v>
       </c>
@@ -4083,7 +4120,7 @@
         <f>AA16</f>
         <v>348</v>
       </c>
-      <c r="J39" s="72">
+      <c r="J39" s="18">
         <f>I39/H39</f>
         <v>0.34017595307917886</v>
       </c>
@@ -4102,11 +4139,11 @@
         <f>D38+D39</f>
         <v>44</v>
       </c>
-      <c r="E40" s="72">
+      <c r="E40" s="18">
         <f>D40/C40</f>
         <v>0.38938053097345132</v>
       </c>
-      <c r="F40" s="74"/>
+      <c r="F40" s="57"/>
       <c r="G40" t="s">
         <v>39</v>
       </c>
@@ -4118,7 +4155,7 @@
         <f>I38+I39</f>
         <v>440</v>
       </c>
-      <c r="J40" s="72">
+      <c r="J40" s="18">
         <f>I40/H40</f>
         <v>0.37963761863675582</v>
       </c>
@@ -4127,18 +4164,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B26:I26"/>
-    <mergeCell ref="B31:I31"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="Q1:T1"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="Q6:T6"/>
     <mergeCell ref="Q12:T12"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B26:I26"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="G20:J20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4150,51 +4187,51 @@
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="7" max="7" width="12.21875" customWidth="1"/>
-    <col min="8" max="8" width="8.77734375" style="37"/>
-    <col min="11" max="11" width="33.21875" style="61" customWidth="1"/>
-    <col min="12" max="12" width="17" style="61" customWidth="1"/>
+    <col min="8" max="8" width="8.77734375"/>
+    <col min="11" max="11" width="33.21875" style="47" customWidth="1"/>
+    <col min="12" max="12" width="17" style="47" customWidth="1"/>
     <col min="13" max="13" width="8.33203125" style="1" customWidth="1"/>
     <col min="14" max="14" width="16.6640625" style="1" customWidth="1"/>
     <col min="15" max="15" width="20.33203125" customWidth="1"/>
-    <col min="16" max="16" width="5.21875" style="52" customWidth="1"/>
+    <col min="16" max="16" width="5.21875" style="40" customWidth="1"/>
     <col min="17" max="17" width="8.77734375" bestFit="1" customWidth="1"/>
     <col min="18" max="19" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="8.77734375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.77734375" style="37"/>
-    <col min="26" max="26" width="33.21875" style="61" customWidth="1"/>
-    <col min="27" max="27" width="17" style="61" customWidth="1"/>
+    <col min="23" max="23" width="8.77734375"/>
+    <col min="26" max="26" width="33.21875" style="47" customWidth="1"/>
+    <col min="27" max="27" width="17" style="47" customWidth="1"/>
     <col min="28" max="28" width="8.33203125" style="1" customWidth="1"/>
     <col min="29" max="29" width="16.6640625" style="1" customWidth="1"/>
     <col min="30" max="30" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="52" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="53" t="s">
+    <row r="1" spans="1:30" s="40" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="Q1" s="53" t="s">
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="Q1" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="53"/>
-      <c r="S1" s="53"/>
-      <c r="T1" s="53"/>
-      <c r="Z1" s="54"/>
-      <c r="AA1" s="54"/>
-      <c r="AB1" s="56"/>
-      <c r="AC1" s="56"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="59"/>
+      <c r="Z1" s="41"/>
+      <c r="AA1" s="41"/>
+      <c r="AB1" s="43"/>
+      <c r="AC1" s="43"/>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -4218,10 +4255,10 @@
         <v>16</v>
       </c>
       <c r="J2" s="3"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="57"/>
-      <c r="N2" s="57"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="20"/>
+      <c r="N2" s="20"/>
       <c r="Q2" s="2" t="s">
         <v>2</v>
       </c>
@@ -4242,10 +4279,10 @@
       <c r="X2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="Z2" s="59"/>
-      <c r="AA2" s="59"/>
-      <c r="AB2" s="57"/>
-      <c r="AC2" s="57"/>
+      <c r="Z2" s="45"/>
+      <c r="AA2" s="45"/>
+      <c r="AB2" s="20"/>
+      <c r="AC2" s="20"/>
     </row>
     <row r="3" spans="1:30" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
@@ -4274,17 +4311,17 @@
         <v>1851.34</v>
       </c>
       <c r="J3" s="14"/>
-      <c r="K3" s="60" t="s">
+      <c r="K3" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="L3" s="67" t="s">
+      <c r="L3" s="53" t="s">
         <v>28</v>
       </c>
       <c r="M3" s="24" t="s">
         <v>30</v>
       </c>
       <c r="N3" s="24"/>
-      <c r="P3" s="52"/>
+      <c r="P3" s="40"/>
       <c r="Q3" s="2">
         <v>138.04</v>
       </c>
@@ -4303,14 +4340,14 @@
       </c>
       <c r="V3" s="2"/>
       <c r="W3" s="2"/>
-      <c r="X3" s="51">
+      <c r="X3" s="39">
         <f>SUM(Q3:R3)</f>
         <v>776.79</v>
       </c>
-      <c r="Z3" s="60" t="s">
+      <c r="Z3" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="AA3" s="67" t="s">
+      <c r="AA3" s="53" t="s">
         <v>28</v>
       </c>
       <c r="AB3" s="24" t="s">
@@ -4328,20 +4365,20 @@
       <c r="H4" s="3"/>
       <c r="I4" s="13"/>
       <c r="J4" s="14"/>
-      <c r="K4" s="60">
+      <c r="K4" s="46">
         <f>B3+D3</f>
         <v>784.78</v>
       </c>
-      <c r="L4" s="60">
+      <c r="L4" s="46">
         <f>B3</f>
         <v>124.05</v>
       </c>
-      <c r="M4" s="65">
+      <c r="M4" s="51">
         <f>L4/K4</f>
         <v>0.15806977751726597</v>
       </c>
-      <c r="N4" s="65"/>
-      <c r="P4" s="52"/>
+      <c r="N4" s="51"/>
+      <c r="P4" s="40"/>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
@@ -4349,20 +4386,20 @@
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
-      <c r="X4" s="51"/>
-      <c r="Z4" s="60">
+      <c r="X4" s="39"/>
+      <c r="Z4" s="46">
         <f>Q3+S3</f>
         <v>667.3</v>
       </c>
-      <c r="AA4" s="60">
+      <c r="AA4" s="46">
         <f>Q3</f>
         <v>138.04</v>
       </c>
-      <c r="AB4" s="65">
+      <c r="AB4" s="51">
         <f>AA4/Z4</f>
         <v>0.20686347969429042</v>
       </c>
-      <c r="AC4" s="65"/>
+      <c r="AC4" s="51"/>
     </row>
     <row r="5" spans="1:30" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B5" s="14"/>
@@ -4371,14 +4408,14 @@
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
-      <c r="H5" s="46"/>
+      <c r="H5" s="14"/>
       <c r="I5" s="27"/>
       <c r="J5" s="14"/>
-      <c r="K5" s="60">
+      <c r="K5" s="46">
         <f>C3+E3</f>
         <v>1786.22</v>
       </c>
-      <c r="L5" s="60">
+      <c r="L5" s="46">
         <f>E3</f>
         <v>58.93</v>
       </c>
@@ -4387,42 +4424,41 @@
         <v>3.2991456819428736E-2</v>
       </c>
       <c r="N5" s="24"/>
-      <c r="P5" s="52"/>
+      <c r="P5" s="40"/>
       <c r="Q5" s="14"/>
       <c r="R5" s="14"/>
       <c r="S5" s="14"/>
       <c r="T5" s="14"/>
       <c r="U5" s="14"/>
-      <c r="W5" s="39"/>
       <c r="X5" s="28"/>
-      <c r="Z5" s="60">
+      <c r="Z5" s="46">
         <f>R3+T3</f>
         <v>663.7</v>
       </c>
-      <c r="AA5" s="60">
+      <c r="AA5" s="46">
         <f>T3</f>
         <v>24.95</v>
       </c>
-      <c r="AB5" s="64">
+      <c r="AB5" s="50">
         <f>AA5/Z5</f>
         <v>3.7592285671237E-2</v>
       </c>
       <c r="AC5" s="24"/>
     </row>
     <row r="6" spans="1:30" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
       <c r="F6" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="36" t="s">
+      <c r="H6" s="13" t="s">
         <v>18</v>
       </c>
       <c r="I6" s="3" t="s">
@@ -4431,26 +4467,26 @@
       <c r="J6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K6" s="67" t="s">
+      <c r="K6" s="53" t="s">
         <v>27</v>
       </c>
       <c r="L6" s="3"/>
-      <c r="M6" s="58"/>
-      <c r="N6" s="58"/>
-      <c r="P6" s="52"/>
-      <c r="Q6" s="33" t="s">
+      <c r="M6" s="44"/>
+      <c r="N6" s="44"/>
+      <c r="P6" s="40"/>
+      <c r="Q6" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="R6" s="33"/>
-      <c r="S6" s="33"/>
-      <c r="T6" s="33"/>
+      <c r="R6" s="60"/>
+      <c r="S6" s="60"/>
+      <c r="T6" s="60"/>
       <c r="U6" s="3" t="s">
         <v>24</v>
       </c>
       <c r="V6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="W6" s="36" t="s">
+      <c r="W6" s="13" t="s">
         <v>18</v>
       </c>
       <c r="X6" s="3" t="s">
@@ -4459,41 +4495,41 @@
       <c r="Y6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="Z6" s="67" t="s">
+      <c r="Z6" s="53" t="s">
         <v>27</v>
       </c>
       <c r="AA6" s="3"/>
-      <c r="AB6" s="58"/>
-      <c r="AC6" s="58"/>
+      <c r="AB6" s="44"/>
+      <c r="AC6" s="44"/>
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H7" s="47"/>
-      <c r="K7" s="61" t="s">
+      <c r="H7" s="20"/>
+      <c r="K7" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="L7" s="67" t="s">
+      <c r="L7" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="M7" s="55" t="s">
+      <c r="M7" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="N7" s="55"/>
+      <c r="N7" s="42"/>
       <c r="R7" s="9"/>
       <c r="S7" s="9"/>
-      <c r="W7" s="47"/>
-      <c r="Z7" s="61" t="s">
+      <c r="W7" s="20"/>
+      <c r="Z7" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="AA7" s="67" t="s">
+      <c r="AA7" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="AB7" s="55" t="s">
+      <c r="AB7" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="AC7" s="55"/>
+      <c r="AC7" s="42"/>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -4519,7 +4555,7 @@
         <f>F8/F3</f>
         <v>0.26876701672500974</v>
       </c>
-      <c r="H8" s="48">
+      <c r="H8" s="38">
         <f>I8/F8</f>
         <v>0.81765557163531111</v>
       </c>
@@ -4531,19 +4567,19 @@
         <f>I8/I3</f>
         <v>0.30518435295515683</v>
       </c>
-      <c r="K8" s="63">
+      <c r="K8" s="49">
         <f>B8+D8</f>
         <v>163</v>
       </c>
-      <c r="L8" s="63">
+      <c r="L8" s="49">
         <f>B8</f>
         <v>43</v>
       </c>
-      <c r="M8" s="65">
+      <c r="M8" s="51">
         <f>L8/K8</f>
         <v>0.26380368098159507</v>
       </c>
-      <c r="N8" s="65"/>
+      <c r="N8" s="51"/>
       <c r="Q8" s="12">
         <v>27</v>
       </c>
@@ -4564,7 +4600,7 @@
         <f>U8/U3</f>
         <v>0.28962434259954922</v>
       </c>
-      <c r="W8" s="40">
+      <c r="W8" s="18">
         <f>X8/U8</f>
         <v>0.78860670834522295</v>
       </c>
@@ -4576,19 +4612,19 @@
         <f>X8/777</f>
         <v>0.39124839124839123</v>
       </c>
-      <c r="Z8" s="63">
+      <c r="Z8" s="49">
         <f>Q8+S8</f>
         <v>104</v>
       </c>
-      <c r="AA8" s="63">
+      <c r="AA8" s="49">
         <f>Q8</f>
         <v>27</v>
       </c>
-      <c r="AB8" s="65">
+      <c r="AB8" s="51">
         <f>AA8/Z8</f>
         <v>0.25961538461538464</v>
       </c>
-      <c r="AC8" s="65"/>
+      <c r="AC8" s="51"/>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -4614,7 +4650,7 @@
         <f>F9/F3</f>
         <v>0.52301050175029185</v>
       </c>
-      <c r="H9" s="48">
+      <c r="H9" s="38">
         <f>I9/F9</f>
         <v>0.80615174096054021</v>
       </c>
@@ -4626,19 +4662,19 @@
         <f>I9/I3</f>
         <v>0.5855218382360885</v>
       </c>
-      <c r="K9" s="63">
+      <c r="K9" s="49">
         <f>B9+D9</f>
         <v>313</v>
       </c>
-      <c r="L9" s="63">
+      <c r="L9" s="49">
         <f>B9</f>
         <v>73</v>
       </c>
-      <c r="M9" s="65">
+      <c r="M9" s="51">
         <f>L9/K9</f>
         <v>0.23322683706070288</v>
       </c>
-      <c r="N9" s="65"/>
+      <c r="N9" s="51"/>
       <c r="Q9" s="12">
         <v>51</v>
       </c>
@@ -4659,7 +4695,7 @@
         <f>U9/U3</f>
         <v>0.46242674680691209</v>
       </c>
-      <c r="W9" s="40">
+      <c r="W9" s="18">
         <f>X9/U9</f>
         <v>0.76524395197322459</v>
       </c>
@@ -4671,19 +4707,19 @@
         <f>X9/777</f>
         <v>0.60617760617760619</v>
       </c>
-      <c r="Z9" s="63">
+      <c r="Z9" s="49">
         <f>Q9+S9</f>
         <v>187</v>
       </c>
-      <c r="AA9" s="63">
+      <c r="AA9" s="49">
         <f>Q9</f>
         <v>51</v>
       </c>
-      <c r="AB9" s="65">
+      <c r="AB9" s="51">
         <f>AA9/Z9</f>
         <v>0.27272727272727271</v>
       </c>
-      <c r="AC9" s="65"/>
+      <c r="AC9" s="51"/>
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -4709,7 +4745,7 @@
         <f>F10/F3</f>
         <v>0.7040062232594323</v>
       </c>
-      <c r="H10" s="48">
+      <c r="H10" s="38">
         <f>I10/F10</f>
         <v>0.77679558011049721</v>
       </c>
@@ -4721,19 +4757,19 @@
         <f>I10/I3</f>
         <v>0.75944991195566458</v>
       </c>
-      <c r="K10" s="63">
+      <c r="K10" s="49">
         <f>B10+D10</f>
         <v>463</v>
       </c>
-      <c r="L10" s="63">
+      <c r="L10" s="49">
         <f>B10</f>
         <v>96</v>
       </c>
-      <c r="M10" s="65">
+      <c r="M10" s="51">
         <f>L10/K10</f>
         <v>0.20734341252699784</v>
       </c>
-      <c r="N10" s="65"/>
+      <c r="N10" s="51"/>
       <c r="Q10" s="12">
         <v>73</v>
       </c>
@@ -4754,7 +4790,7 @@
         <f>U10/U3</f>
         <v>0.54845980465815181</v>
       </c>
-      <c r="W10" s="40">
+      <c r="W10" s="18">
         <f>X10/U10</f>
         <v>0.7</v>
       </c>
@@ -4766,65 +4802,65 @@
         <f>X10/777</f>
         <v>0.65765765765765771</v>
       </c>
-      <c r="Z10" s="63">
+      <c r="Z10" s="49">
         <f>Q10+S10</f>
         <v>284</v>
       </c>
-      <c r="AA10" s="63">
+      <c r="AA10" s="49">
         <f>Q10</f>
         <v>73</v>
       </c>
-      <c r="AB10" s="65">
+      <c r="AB10" s="51">
         <f>AA10/Z10</f>
         <v>0.25704225352112675</v>
       </c>
-      <c r="AC10" s="65"/>
+      <c r="AC10" s="51"/>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.35">
       <c r="F11" s="11"/>
       <c r="G11" s="15"/>
-      <c r="H11" s="48"/>
+      <c r="H11" s="38"/>
       <c r="I11" s="15"/>
       <c r="J11" s="15"/>
-      <c r="K11" s="62"/>
-      <c r="L11" s="62"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="48"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
       <c r="U11" s="11"/>
-      <c r="Z11" s="62"/>
-      <c r="AA11" s="62"/>
+      <c r="Z11" s="48"/>
+      <c r="AA11" s="48"/>
       <c r="AB11" s="8"/>
       <c r="AC11" s="8"/>
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
+      <c r="C12" s="58"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="58"/>
       <c r="F12" s="11"/>
       <c r="G12" s="15"/>
-      <c r="H12" s="48"/>
+      <c r="H12" s="38"/>
       <c r="I12" s="15"/>
       <c r="J12" s="15"/>
-      <c r="K12" s="63" t="s">
+      <c r="K12" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="L12" s="63"/>
+      <c r="L12" s="49"/>
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
-      <c r="Q12" s="34" t="s">
+      <c r="Q12" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="R12" s="34"/>
-      <c r="S12" s="34"/>
-      <c r="T12" s="34"/>
+      <c r="R12" s="58"/>
+      <c r="S12" s="58"/>
+      <c r="T12" s="58"/>
       <c r="U12" s="11"/>
-      <c r="Z12" s="63" t="s">
+      <c r="Z12" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="AA12" s="63"/>
+      <c r="AA12" s="49"/>
       <c r="AB12" s="8"/>
       <c r="AC12" s="8"/>
     </row>
@@ -4838,21 +4874,21 @@
       <c r="E13" s="9"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
-      <c r="H13" s="36"/>
+      <c r="H13" s="13"/>
       <c r="I13" s="13">
         <f>SUM(D3:E3)</f>
         <v>719.66</v>
       </c>
-      <c r="K13" s="61" t="s">
+      <c r="K13" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="L13" s="67" t="s">
+      <c r="L13" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="M13" s="55" t="s">
+      <c r="M13" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="N13" s="68" t="s">
+      <c r="N13" s="54" t="s">
         <v>32</v>
       </c>
       <c r="O13" s="11" t="s">
@@ -4868,16 +4904,16 @@
         <f>SUM(S3:T3)</f>
         <v>554.21</v>
       </c>
-      <c r="Z13" s="61" t="s">
+      <c r="Z13" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="AA13" s="67" t="s">
+      <c r="AA13" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="AB13" s="55" t="s">
+      <c r="AB13" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="AC13" s="68" t="s">
+      <c r="AC13" s="54" t="s">
         <v>32</v>
       </c>
       <c r="AD13" s="11" t="s">
@@ -4888,11 +4924,11 @@
       <c r="A14" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="49">
+      <c r="B14" s="7">
         <f>B3-B8</f>
         <v>81.05</v>
       </c>
-      <c r="C14" s="49">
+      <c r="C14" s="7">
         <f>C3-C8</f>
         <v>1205.29</v>
       </c>
@@ -4912,7 +4948,7 @@
         <f>F14/F3</f>
         <v>0.73123298327499042</v>
       </c>
-      <c r="H14" s="38">
+      <c r="H14" s="33">
         <f>I14/F14</f>
         <v>0.31577659574468081</v>
       </c>
@@ -4932,23 +4968,23 @@
         <f>B14+E14</f>
         <v>133.97999999999999</v>
       </c>
-      <c r="M14" s="66">
+      <c r="M14" s="52">
         <f>L14/K14</f>
         <v>7.1265957446808512E-2</v>
       </c>
-      <c r="N14" s="69">
-        <f>K8+K14</f>
+      <c r="N14" s="55">
+        <f t="shared" ref="N14:O16" si="1">K8+K14</f>
         <v>2043</v>
       </c>
       <c r="O14" s="14">
-        <f>L8+L14</f>
+        <f t="shared" si="1"/>
         <v>176.98</v>
       </c>
-      <c r="Q14" s="49">
+      <c r="Q14" s="7">
         <f>Q3-Q8</f>
         <v>111.03999999999999</v>
       </c>
-      <c r="R14" s="49">
+      <c r="R14" s="7">
         <f>R3-R8</f>
         <v>361.75</v>
       </c>
@@ -4968,7 +5004,7 @@
         <f>U14/U3</f>
         <v>0.71037565740045083</v>
       </c>
-      <c r="W14" s="41">
+      <c r="W14" s="34">
         <f>X14/U14</f>
         <v>0.49996298294042368</v>
       </c>
@@ -4988,16 +5024,16 @@
         <f>Q14+T14</f>
         <v>131.5</v>
       </c>
-      <c r="AB14" s="66">
+      <c r="AB14" s="52">
         <f>AA14/Z14</f>
         <v>0.13907838097957717</v>
       </c>
-      <c r="AC14" s="69">
-        <f>Z8+Z14</f>
+      <c r="AC14" s="55">
+        <f t="shared" ref="AC14:AD16" si="2">Z8+Z14</f>
         <v>1049.51</v>
       </c>
       <c r="AD14" s="14">
-        <f>AA8+AA14</f>
+        <f t="shared" si="2"/>
         <v>158.5</v>
       </c>
     </row>
@@ -5029,7 +5065,7 @@
         <f>F15/F3</f>
         <v>0.47698949824970832</v>
       </c>
-      <c r="H15" s="38">
+      <c r="H15" s="33">
         <f>I15/F15</f>
         <v>0.37428445618670192</v>
       </c>
@@ -5049,16 +5085,16 @@
         <f>B15+E15</f>
         <v>89.32</v>
       </c>
-      <c r="M15" s="66">
+      <c r="M15" s="52">
         <f>L15/K15</f>
         <v>7.2834613565569098E-2</v>
       </c>
-      <c r="N15" s="69">
-        <f>K9+K15</f>
+      <c r="N15" s="55">
+        <f t="shared" si="1"/>
         <v>1539.34</v>
       </c>
       <c r="O15" s="14">
-        <f>L9+L15</f>
+        <f t="shared" si="1"/>
         <v>162.32</v>
       </c>
       <c r="Q15" s="7">
@@ -5085,7 +5121,7 @@
         <f>U15/U3</f>
         <v>0.53757325319308791</v>
       </c>
-      <c r="W15" s="41">
+      <c r="W15" s="34">
         <f>X15/U15</f>
         <v>0.57262651814789445</v>
       </c>
@@ -5105,16 +5141,16 @@
         <f>Q15+T15</f>
         <v>103.5</v>
       </c>
-      <c r="AB15" s="66">
+      <c r="AB15" s="52">
         <f>AA15/Z15</f>
         <v>0.14465206635826194</v>
       </c>
-      <c r="AC15" s="69">
-        <f>Z9+Z15</f>
+      <c r="AC15" s="55">
+        <f t="shared" si="2"/>
         <v>902.51</v>
       </c>
       <c r="AD15" s="14">
-        <f>AA9+AA15</f>
+        <f t="shared" si="2"/>
         <v>154.5</v>
       </c>
     </row>
@@ -5146,7 +5182,7 @@
         <f>F16/F3</f>
         <v>0.29599377674056787</v>
       </c>
-      <c r="H16" s="38">
+      <c r="H16" s="33">
         <f>I16/F16</f>
         <v>0.41479632063074912</v>
       </c>
@@ -5166,16 +5202,16 @@
         <f>B16+E16</f>
         <v>49.98</v>
       </c>
-      <c r="M16" s="66">
+      <c r="M16" s="52">
         <f>L16/K16</f>
         <v>6.567674113009199E-2</v>
       </c>
-      <c r="N16" s="69">
-        <f>K10+K16</f>
+      <c r="N16" s="55">
+        <f t="shared" si="1"/>
         <v>1224</v>
       </c>
       <c r="O16" s="14">
-        <f>L10+L16</f>
+        <f t="shared" si="1"/>
         <v>145.97999999999999</v>
       </c>
       <c r="Q16" s="7">
@@ -5202,7 +5238,7 @@
         <f>U16/U3</f>
         <v>0.45154019534184825</v>
       </c>
-      <c r="W16" s="41">
+      <c r="W16" s="34">
         <f>X16/U16</f>
         <v>0.55775374376039932</v>
       </c>
@@ -5222,44 +5258,47 @@
         <f>Q16+T16</f>
         <v>81.99</v>
       </c>
-      <c r="AB16" s="66">
+      <c r="AB16" s="52">
         <f>AA16/Z16</f>
         <v>0.13642262895174709</v>
       </c>
-      <c r="AC16" s="69">
-        <f>Z10+Z16</f>
+      <c r="AC16" s="55">
+        <f t="shared" si="2"/>
         <v>885</v>
       </c>
       <c r="AD16" s="14">
-        <f>AA10+AA16</f>
+        <f t="shared" si="2"/>
         <v>154.99</v>
       </c>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B20" s="11"/>
-      <c r="C20" s="34" t="s">
-        <v>0</v>
-      </c>
-      <c r="D20" s="34"/>
-      <c r="E20" s="11"/>
-      <c r="H20" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="I20" s="34"/>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B21" s="34" t="s">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B20" s="58" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="58"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="58"/>
+      <c r="G20" s="58" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" s="58"/>
+      <c r="I20" s="58"/>
+      <c r="J20" s="58"/>
+      <c r="K20" s="62"/>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B21" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
-    </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="C21" s="58"/>
+      <c r="D21" s="58"/>
+      <c r="E21" s="58"/>
+      <c r="F21" s="58"/>
+      <c r="G21" s="58"/>
+      <c r="H21" s="58"/>
+      <c r="I21" s="58"/>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B22" s="11" t="s">
         <v>38</v>
       </c>
@@ -5267,12 +5306,12 @@
         <v>36</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F22" s="73"/>
+      <c r="F22" s="56"/>
       <c r="G22" s="11" t="s">
         <v>38</v>
       </c>
@@ -5280,46 +5319,46 @@
         <v>36</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J22" s="11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B23" s="70">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B23">
         <v>1</v>
       </c>
-      <c r="C23" s="71">
+      <c r="C23" s="9">
         <f>K4</f>
         <v>784.78</v>
       </c>
-      <c r="D23" s="71">
+      <c r="D23" s="9">
         <f>L4</f>
         <v>124.05</v>
       </c>
-      <c r="E23" s="72">
+      <c r="E23" s="18">
         <f>D23/C23</f>
         <v>0.15806977751726597</v>
       </c>
-      <c r="F23" s="73"/>
-      <c r="G23" s="70">
+      <c r="F23" s="56"/>
+      <c r="G23">
         <v>1</v>
       </c>
-      <c r="H23" s="71">
+      <c r="H23" s="9">
         <f>Z4</f>
         <v>667.3</v>
       </c>
-      <c r="I23" s="71">
+      <c r="I23" s="9">
         <f>AA4</f>
         <v>138.04</v>
       </c>
-      <c r="J23" s="72">
+      <c r="J23" s="18">
         <f>I23/H23</f>
         <v>0.20686347969429042</v>
       </c>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B24">
         <v>2</v>
       </c>
@@ -5331,11 +5370,11 @@
         <f>L5</f>
         <v>58.93</v>
       </c>
-      <c r="E24" s="72">
+      <c r="E24" s="18">
         <f>D24/C24</f>
         <v>3.2991456819428736E-2</v>
       </c>
-      <c r="F24" s="74"/>
+      <c r="F24" s="57"/>
       <c r="G24">
         <v>2</v>
       </c>
@@ -5347,12 +5386,12 @@
         <f>AA5</f>
         <v>24.95</v>
       </c>
-      <c r="J24" s="72">
+      <c r="J24" s="18">
         <f>I24/H24</f>
         <v>3.7592285671237E-2</v>
       </c>
     </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>39</v>
       </c>
@@ -5364,11 +5403,11 @@
         <f>D23+D24</f>
         <v>182.98</v>
       </c>
-      <c r="E25" s="72">
+      <c r="E25" s="18">
         <f>D25/C25</f>
         <v>7.1170750680668998E-2</v>
       </c>
-      <c r="F25" s="74"/>
+      <c r="F25" s="57"/>
       <c r="G25" t="s">
         <v>39</v>
       </c>
@@ -5380,24 +5419,24 @@
         <f>I23+I24</f>
         <v>162.98999999999998</v>
       </c>
-      <c r="J25" s="72">
+      <c r="J25" s="18">
         <f>I25/H25</f>
         <v>0.12245679939894814</v>
       </c>
     </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B26" s="32" t="s">
+    <row r="26" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B26" s="61" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="32"/>
-    </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="C26" s="61"/>
+      <c r="D26" s="61"/>
+      <c r="E26" s="61"/>
+      <c r="F26" s="61"/>
+      <c r="G26" s="61"/>
+      <c r="H26" s="61"/>
+      <c r="I26" s="61"/>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B27" s="11" t="s">
         <v>38</v>
       </c>
@@ -5417,7 +5456,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B28">
         <v>1</v>
       </c>
@@ -5429,11 +5468,11 @@
         <f>L8</f>
         <v>43</v>
       </c>
-      <c r="E28" s="72">
+      <c r="E28" s="18">
         <f>D28/C28</f>
         <v>0.26380368098159507</v>
       </c>
-      <c r="F28" s="74"/>
+      <c r="F28" s="57"/>
       <c r="G28">
         <v>1</v>
       </c>
@@ -5445,12 +5484,12 @@
         <f>AA8</f>
         <v>27</v>
       </c>
-      <c r="J28" s="72">
+      <c r="J28" s="18">
         <f>I28/H28</f>
         <v>0.25961538461538464</v>
       </c>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B29">
         <v>2</v>
       </c>
@@ -5462,11 +5501,11 @@
         <f>L14</f>
         <v>133.97999999999999</v>
       </c>
-      <c r="E29" s="72">
+      <c r="E29" s="18">
         <f>D29/C29</f>
         <v>7.1265957446808512E-2</v>
       </c>
-      <c r="F29" s="74"/>
+      <c r="F29" s="57"/>
       <c r="G29">
         <v>2</v>
       </c>
@@ -5478,12 +5517,12 @@
         <f>AA14</f>
         <v>131.5</v>
       </c>
-      <c r="J29" s="72">
+      <c r="J29" s="18">
         <f>I29/H29</f>
         <v>0.13907838097957717</v>
       </c>
     </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>39</v>
       </c>
@@ -5495,11 +5534,11 @@
         <f>D28+D29</f>
         <v>176.98</v>
       </c>
-      <c r="E30" s="72">
+      <c r="E30" s="18">
         <f>D30/C30</f>
         <v>8.6627508565834552E-2</v>
       </c>
-      <c r="F30" s="74"/>
+      <c r="F30" s="57"/>
       <c r="G30" t="s">
         <v>39</v>
       </c>
@@ -5511,24 +5550,24 @@
         <f>I28+I29</f>
         <v>158.5</v>
       </c>
-      <c r="J30" s="72">
+      <c r="J30" s="18">
         <f>I30/H30</f>
         <v>0.15102285828624787</v>
       </c>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B31" s="32" t="s">
+    <row r="31" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B31" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="32"/>
-    </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="C31" s="61"/>
+      <c r="D31" s="61"/>
+      <c r="E31" s="61"/>
+      <c r="F31" s="61"/>
+      <c r="G31" s="61"/>
+      <c r="H31" s="61"/>
+      <c r="I31" s="61"/>
+    </row>
+    <row r="32" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B32" s="11" t="s">
         <v>38</v>
       </c>
@@ -5560,11 +5599,11 @@
         <f>L9</f>
         <v>73</v>
       </c>
-      <c r="E33" s="72">
+      <c r="E33" s="18">
         <f>D33/C33</f>
         <v>0.23322683706070288</v>
       </c>
-      <c r="F33" s="74"/>
+      <c r="F33" s="57"/>
       <c r="G33">
         <v>1</v>
       </c>
@@ -5576,7 +5615,7 @@
         <f>AA9</f>
         <v>51</v>
       </c>
-      <c r="J33" s="72">
+      <c r="J33" s="18">
         <f>I33/H33</f>
         <v>0.27272727272727271</v>
       </c>
@@ -5593,11 +5632,11 @@
         <f>L15</f>
         <v>89.32</v>
       </c>
-      <c r="E34" s="72">
+      <c r="E34" s="18">
         <f>D34/C34</f>
         <v>7.2834613565569098E-2</v>
       </c>
-      <c r="F34" s="74"/>
+      <c r="F34" s="57"/>
       <c r="G34">
         <v>2</v>
       </c>
@@ -5609,7 +5648,7 @@
         <f>AA15</f>
         <v>103.5</v>
       </c>
-      <c r="J34" s="72">
+      <c r="J34" s="18">
         <f>I34/H34</f>
         <v>0.14465206635826194</v>
       </c>
@@ -5626,11 +5665,11 @@
         <f>D33+D34</f>
         <v>162.32</v>
       </c>
-      <c r="E35" s="72">
+      <c r="E35" s="18">
         <f>D35/C35</f>
         <v>0.10544778931230267</v>
       </c>
-      <c r="F35" s="74"/>
+      <c r="F35" s="57"/>
       <c r="G35" t="s">
         <v>39</v>
       </c>
@@ -5642,22 +5681,22 @@
         <f>I33+I34</f>
         <v>154.5</v>
       </c>
-      <c r="J35" s="72">
+      <c r="J35" s="18">
         <f>I35/H35</f>
         <v>0.1711892389004</v>
       </c>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B36" s="32" t="s">
+      <c r="B36" s="61" t="s">
         <v>42</v>
       </c>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-      <c r="H36" s="32"/>
-      <c r="I36" s="32"/>
+      <c r="C36" s="61"/>
+      <c r="D36" s="61"/>
+      <c r="E36" s="61"/>
+      <c r="F36" s="61"/>
+      <c r="G36" s="61"/>
+      <c r="H36" s="61"/>
+      <c r="I36" s="61"/>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B37" s="11" t="s">
@@ -5691,11 +5730,11 @@
         <f>L10</f>
         <v>96</v>
       </c>
-      <c r="E38" s="72">
+      <c r="E38" s="18">
         <f>D38/C38</f>
         <v>0.20734341252699784</v>
       </c>
-      <c r="F38" s="74"/>
+      <c r="F38" s="57"/>
       <c r="G38">
         <v>1</v>
       </c>
@@ -5707,7 +5746,7 @@
         <f>AA10</f>
         <v>73</v>
       </c>
-      <c r="J38" s="72">
+      <c r="J38" s="18">
         <f>I38/H38</f>
         <v>0.25704225352112675</v>
       </c>
@@ -5724,11 +5763,11 @@
         <f>L16</f>
         <v>49.98</v>
       </c>
-      <c r="E39" s="72">
+      <c r="E39" s="18">
         <f>D39/C39</f>
         <v>6.567674113009199E-2</v>
       </c>
-      <c r="F39" s="74"/>
+      <c r="F39" s="57"/>
       <c r="G39">
         <v>2</v>
       </c>
@@ -5740,7 +5779,7 @@
         <f>AA16</f>
         <v>81.99</v>
       </c>
-      <c r="J39" s="72">
+      <c r="J39" s="18">
         <f>I39/H39</f>
         <v>0.13642262895174709</v>
       </c>
@@ -5757,11 +5796,11 @@
         <f>D38+D39</f>
         <v>145.97999999999999</v>
       </c>
-      <c r="E40" s="72">
+      <c r="E40" s="18">
         <f>D40/C40</f>
         <v>0.11926470588235294</v>
       </c>
-      <c r="F40" s="74"/>
+      <c r="F40" s="57"/>
       <c r="G40" t="s">
         <v>39</v>
       </c>
@@ -5773,18 +5812,13 @@
         <f>I38+I39</f>
         <v>154.99</v>
       </c>
-      <c r="J40" s="72">
+      <c r="J40" s="18">
         <f>I40/H40</f>
         <v>0.17512994350282488</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B26:I26"/>
-    <mergeCell ref="B31:I31"/>
     <mergeCell ref="B36:I36"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="Q1:T1"/>
@@ -5792,6 +5826,11 @@
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="Q12:T12"/>
     <mergeCell ref="Q6:T6"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B26:I26"/>
+    <mergeCell ref="B31:I31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>